<commit_message>
Actualización de archivos JSON y scripts 17 de marzo 2026
</commit_message>
<xml_diff>
--- a/Tuya.xlsx
+++ b/Tuya.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Hoja2" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'EN PROCESO (Tuya)'!$A$1:$AN$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'EN PROCESO (Tuya)'!$A$1:$AN$106</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="776" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="383">
   <si>
     <t>Asignado a</t>
   </si>
@@ -1193,7 +1193,26 @@
     <t>el cliente solicita a imagine en sala azul para revisar incidente de afectacion general en las dematerialización de pagares</t>
   </si>
   <si>
-    <t>EN PROCESO</t>
+    <t>09/03/2026: Se realiza el acompañamineto por parte de Imagine, se realizan todas las validaciones y se descarta fallas de nuestro aplicativo, se entregan evidencias de los errores de consumo del servicio de pagare el cual es de otro proveedor.</t>
+  </si>
+  <si>
+    <t>363</t>
+  </si>
+  <si>
+    <t>12/03/2026: Se realiza la validación del caso y se da solución al usuario.</t>
+  </si>
+  <si>
+    <t>364</t>
+  </si>
+  <si>
+    <t>Validación con cliente</t>
+  </si>
+  <si>
+    <t>Agendamiento para contingencia</t>
+  </si>
+  <si>
+    <t>16/03/2026: Cliente se comunica para validar disponibilidad para agendamiento de proceso contingencia, se esta a la espera del email por parte de ellos
+17/03/2026: Notifican agendamiento prueba de continuidad para el 24/03/2026</t>
   </si>
   <si>
     <t xml:space="preserve"> Año Nuevo</t>
@@ -1746,7 +1765,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="141">
+  <cellXfs count="139">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2135,12 +2154,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="14" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -2375,7 +2388,7 @@
   <sheetPr>
     <tabColor rgb="FF93C47D"/>
   </sheetPr>
-  <dimension ref="A1:AN104"/>
+  <dimension ref="A1:AN106"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.21875" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -2514,7 +2527,7 @@
       NETWORKDAYS(J2,L2,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="N2" s="21"/>
       <c r="O2" s="21"/>
@@ -2583,7 +2596,7 @@
       NETWORKDAYS(J3,L3,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="N3" s="34"/>
       <c r="O3" s="34"/>
@@ -2654,7 +2667,7 @@
       NETWORKDAYS(J4,L4,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="N4" s="22"/>
       <c r="O4" s="22"/>
@@ -2725,7 +2738,7 @@
       NETWORKDAYS(J5,L5,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="N5" s="34"/>
       <c r="O5" s="34"/>
@@ -2796,7 +2809,7 @@
       NETWORKDAYS(J6,L6,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="N6" s="21"/>
       <c r="O6" s="21"/>
@@ -2867,7 +2880,7 @@
       NETWORKDAYS(J7,L7,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="N7" s="41"/>
       <c r="O7" s="41"/>
@@ -2938,7 +2951,7 @@
       NETWORKDAYS(J8,L8,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="N8" s="22"/>
       <c r="O8" s="22"/>
@@ -3599,7 +3612,7 @@
       NETWORKDAYS(J17,L17,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="N17" s="35"/>
       <c r="O17" s="35"/>
@@ -4911,7 +4924,7 @@
       NETWORKDAYS(J35,L35,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="N35" s="76"/>
       <c r="O35" s="76">
@@ -5497,7 +5510,7 @@
       NETWORKDAYS(J43,L43,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="N43" s="41"/>
       <c r="O43" s="41"/>
@@ -9489,7 +9502,7 @@
       <c r="O97" s="41"/>
       <c r="P97" s="41"/>
       <c r="Q97" s="92"/>
-      <c r="R97" s="137" t="s">
+      <c r="R97" s="133" t="s">
         <v>39</v>
       </c>
       <c r="S97" s="113"/>
@@ -9868,7 +9881,9 @@
         <v>46091</v>
       </c>
       <c r="O102" s="44"/>
-      <c r="P102" s="44"/>
+      <c r="P102" s="68">
+        <v>46087</v>
+      </c>
       <c r="Q102" s="128" t="s">
         <v>330</v>
       </c>
@@ -9990,7 +10005,7 @@
       </c>
       <c r="E104" s="93"/>
       <c r="F104" s="103" t="s">
-        <v>339</v>
+        <v>46</v>
       </c>
       <c r="G104" s="104">
         <v>100</v>
@@ -10006,7 +10021,9 @@
         <v>46090</v>
       </c>
       <c r="K104" s="44"/>
-      <c r="L104" s="44"/>
+      <c r="L104" s="68">
+        <v>46090</v>
+      </c>
       <c r="M104" s="23">
         <f ca="1">IF(OR(J104="",AND(L104="",TODAY()&lt;J104),AND(L104&lt;&gt;"",L104&lt;J104)),0,
    IF(L104="",
@@ -10019,8 +10036,12 @@
       <c r="N104" s="44"/>
       <c r="O104" s="44"/>
       <c r="P104" s="44"/>
-      <c r="Q104" s="136"/>
-      <c r="R104" s="137"/>
+      <c r="Q104" s="128" t="s">
+        <v>339</v>
+      </c>
+      <c r="R104" s="129" t="s">
+        <v>39</v>
+      </c>
       <c r="S104" s="117"/>
       <c r="T104" s="118"/>
       <c r="U104" s="118"/>
@@ -10044,18 +10065,168 @@
       <c r="AM104" s="118"/>
       <c r="AN104" s="119"/>
     </row>
+    <row r="105" spans="1:40">
+      <c r="A105" s="112" t="s">
+        <v>287</v>
+      </c>
+      <c r="B105" s="130" t="s">
+        <v>340</v>
+      </c>
+      <c r="C105" s="84" t="s">
+        <v>204</v>
+      </c>
+      <c r="D105" s="90" t="s">
+        <v>211</v>
+      </c>
+      <c r="E105" s="95"/>
+      <c r="F105" s="101" t="s">
+        <v>46</v>
+      </c>
+      <c r="G105" s="102">
+        <v>100</v>
+      </c>
+      <c r="H105" s="33">
+        <f>IF(OR(J105="",K105="",K105&lt;J105),0,NETWORKDAYS(J105,K105,Hoja2!$A$2:$A$53))</f>
+        <v>1</v>
+      </c>
+      <c r="I105" s="76">
+        <v>46092</v>
+      </c>
+      <c r="J105" s="76">
+        <v>46093</v>
+      </c>
+      <c r="K105" s="76">
+        <v>46093</v>
+      </c>
+      <c r="L105" s="76">
+        <v>46093</v>
+      </c>
+      <c r="M105" s="36">
+        <f ca="1">IF(OR(J105="",AND(L105="",TODAY()&lt;J105),AND(L105&lt;&gt;"",L105&lt;J105)),0,
+   IF(L105="",
+      NETWORKDAYS(J105,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J105,L105,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N105" s="41"/>
+      <c r="O105" s="41"/>
+      <c r="P105" s="41"/>
+      <c r="Q105" s="92" t="s">
+        <v>341</v>
+      </c>
+      <c r="R105" s="133" t="s">
+        <v>39</v>
+      </c>
+      <c r="S105" s="113"/>
+      <c r="T105" s="114"/>
+      <c r="U105" s="114"/>
+      <c r="V105" s="114"/>
+      <c r="W105" s="114"/>
+      <c r="X105" s="114"/>
+      <c r="Y105" s="114"/>
+      <c r="Z105" s="114"/>
+      <c r="AA105" s="114"/>
+      <c r="AB105" s="114"/>
+      <c r="AC105" s="114"/>
+      <c r="AD105" s="114"/>
+      <c r="AE105" s="114"/>
+      <c r="AF105" s="114"/>
+      <c r="AG105" s="114"/>
+      <c r="AH105" s="114"/>
+      <c r="AI105" s="114"/>
+      <c r="AJ105" s="114"/>
+      <c r="AK105" s="114"/>
+      <c r="AL105" s="114"/>
+      <c r="AM105" s="114"/>
+      <c r="AN105" s="115"/>
+    </row>
+    <row r="106" spans="1:40">
+      <c r="A106" s="116" t="s">
+        <v>287</v>
+      </c>
+      <c r="B106" s="134" t="s">
+        <v>342</v>
+      </c>
+      <c r="C106" s="87" t="s">
+        <v>343</v>
+      </c>
+      <c r="D106" s="91" t="s">
+        <v>344</v>
+      </c>
+      <c r="E106" s="93"/>
+      <c r="F106" s="103" t="s">
+        <v>251</v>
+      </c>
+      <c r="G106" s="104">
+        <v>0</v>
+      </c>
+      <c r="H106" s="20">
+        <f>IF(OR(J106="",K106="",K106&lt;J106),0,NETWORKDAYS(J106,K106,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I106" s="68">
+        <v>46097</v>
+      </c>
+      <c r="J106" s="68">
+        <v>46105</v>
+      </c>
+      <c r="K106" s="68"/>
+      <c r="L106" s="68"/>
+      <c r="M106" s="23">
+        <f ca="1">IF(OR(J106="",AND(L106="",TODAY()&lt;J106),AND(L106&lt;&gt;"",L106&lt;J106)),0,
+   IF(L106="",
+      NETWORKDAYS(J106,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J106,L106,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
+      </c>
+      <c r="N106" s="44"/>
+      <c r="O106" s="44"/>
+      <c r="P106" s="44"/>
+      <c r="Q106" s="128" t="s">
+        <v>345</v>
+      </c>
+      <c r="R106" s="129" t="s">
+        <v>39</v>
+      </c>
+      <c r="S106" s="117"/>
+      <c r="T106" s="118"/>
+      <c r="U106" s="118"/>
+      <c r="V106" s="118"/>
+      <c r="W106" s="118"/>
+      <c r="X106" s="118"/>
+      <c r="Y106" s="118"/>
+      <c r="Z106" s="118"/>
+      <c r="AA106" s="118"/>
+      <c r="AB106" s="118"/>
+      <c r="AC106" s="118"/>
+      <c r="AD106" s="118"/>
+      <c r="AE106" s="118"/>
+      <c r="AF106" s="118"/>
+      <c r="AG106" s="118"/>
+      <c r="AH106" s="118"/>
+      <c r="AI106" s="118"/>
+      <c r="AJ106" s="118"/>
+      <c r="AK106" s="118"/>
+      <c r="AL106" s="118"/>
+      <c r="AM106" s="118"/>
+      <c r="AN106" s="119"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AN104"/>
-  <conditionalFormatting sqref="B2:B104">
+  <autoFilter ref="A1:AN106"/>
+  <conditionalFormatting sqref="B2:B106">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>COUNTIF(B$2:B$16,B2)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="I2:L9 J10:L10 I11:L54 N2:P54 I56:L104 N56:P104">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="I2:L9 J10:L10 I11:L54 N2:P54 I56:L106 N56:P106">
       <formula1>OR(NOT(ISERROR(DATEVALUE(I2))), AND(ISNUMBER(I2), LEFT(CELL("format", I2))="D"))</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F104">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F106">
       <formula1>"FINALIZADO,EN PROCESO,PAUSADO,EN TEST,PENDIENTE,PRUEBAS CLIENTE,PRUEBAS IMAGINE,PASO A PRODUCCION"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10073,427 +10244,427 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A1" s="138">
+      <c r="A1" s="136">
         <v>45292</v>
       </c>
-      <c r="B1" s="139" t="s">
-        <v>340</v>
+      <c r="B1" s="137" t="s">
+        <v>346</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A2" s="138">
+      <c r="A2" s="136">
         <v>45299</v>
       </c>
-      <c r="B2" s="139" t="s">
-        <v>341</v>
+      <c r="B2" s="137" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A3" s="138">
+      <c r="A3" s="136">
         <v>45376</v>
       </c>
-      <c r="B3" s="139" t="s">
-        <v>342</v>
+      <c r="B3" s="137" t="s">
+        <v>348</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A4" s="138">
+      <c r="A4" s="136">
         <v>45379</v>
       </c>
-      <c r="B4" s="139" t="s">
-        <v>343</v>
+      <c r="B4" s="137" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A5" s="138">
+      <c r="A5" s="136">
         <v>45380</v>
       </c>
-      <c r="B5" s="139" t="s">
-        <v>344</v>
+      <c r="B5" s="137" t="s">
+        <v>350</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A6" s="138">
+      <c r="A6" s="136">
         <v>45413</v>
       </c>
-      <c r="B6" s="139" t="s">
-        <v>345</v>
+      <c r="B6" s="137" t="s">
+        <v>351</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A7" s="138">
+      <c r="A7" s="136">
         <v>45425</v>
       </c>
-      <c r="B7" s="139" t="s">
-        <v>346</v>
+      <c r="B7" s="137" t="s">
+        <v>352</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A8" s="138">
+      <c r="A8" s="136">
         <v>45446</v>
       </c>
-      <c r="B8" s="139" t="s">
-        <v>347</v>
+      <c r="B8" s="137" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A9" s="138">
+      <c r="A9" s="136">
         <v>45453</v>
       </c>
-      <c r="B9" s="139" t="s">
-        <v>348</v>
+      <c r="B9" s="137" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A10" s="138">
+      <c r="A10" s="136">
         <v>45474</v>
       </c>
-      <c r="B10" s="139" t="s">
-        <v>349</v>
+      <c r="B10" s="137" t="s">
+        <v>355</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A11" s="138">
+      <c r="A11" s="136">
         <v>45493</v>
       </c>
-      <c r="B11" s="139" t="s">
-        <v>350</v>
+      <c r="B11" s="137" t="s">
+        <v>356</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A12" s="138">
+      <c r="A12" s="136">
         <v>45511</v>
       </c>
-      <c r="B12" s="139" t="s">
-        <v>351</v>
+      <c r="B12" s="137" t="s">
+        <v>357</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A13" s="138">
+      <c r="A13" s="136">
         <v>45523</v>
       </c>
-      <c r="B13" s="139" t="s">
-        <v>352</v>
+      <c r="B13" s="137" t="s">
+        <v>358</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A14" s="138">
+      <c r="A14" s="136">
         <v>45579</v>
       </c>
-      <c r="B14" s="139" t="s">
-        <v>353</v>
+      <c r="B14" s="137" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A15" s="138">
+      <c r="A15" s="136">
         <v>45600</v>
       </c>
-      <c r="B15" s="139" t="s">
-        <v>354</v>
+      <c r="B15" s="137" t="s">
+        <v>360</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A16" s="138">
+      <c r="A16" s="136">
         <v>45607</v>
       </c>
-      <c r="B16" s="139" t="s">
-        <v>355</v>
+      <c r="B16" s="137" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A17" s="138">
+      <c r="A17" s="136">
         <v>45634</v>
       </c>
-      <c r="B17" s="139" t="s">
-        <v>356</v>
+      <c r="B17" s="137" t="s">
+        <v>362</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A18" s="138">
+      <c r="A18" s="136">
         <v>45651</v>
       </c>
-      <c r="B18" s="139" t="s">
-        <v>357</v>
+      <c r="B18" s="137" t="s">
+        <v>363</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A19" s="138">
+      <c r="A19" s="136">
         <v>45658</v>
       </c>
-      <c r="B19" s="140" t="s">
-        <v>358</v>
+      <c r="B19" s="138" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A20" s="138">
+      <c r="A20" s="136">
         <v>45663</v>
       </c>
-      <c r="B20" s="140" t="s">
-        <v>359</v>
+      <c r="B20" s="138" t="s">
+        <v>365</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A21" s="138">
+      <c r="A21" s="136">
         <v>45740</v>
       </c>
-      <c r="B21" s="140" t="s">
-        <v>360</v>
+      <c r="B21" s="138" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A22" s="138">
+      <c r="A22" s="136">
         <v>45764</v>
       </c>
-      <c r="B22" s="140" t="s">
-        <v>361</v>
+      <c r="B22" s="138" t="s">
+        <v>367</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A23" s="138">
+      <c r="A23" s="136">
         <v>45765</v>
       </c>
-      <c r="B23" s="140" t="s">
-        <v>362</v>
+      <c r="B23" s="138" t="s">
+        <v>368</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A24" s="138">
+      <c r="A24" s="136">
         <v>45778</v>
       </c>
-      <c r="B24" s="140" t="s">
-        <v>363</v>
+      <c r="B24" s="138" t="s">
+        <v>369</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A25" s="138">
+      <c r="A25" s="136">
         <v>45810</v>
       </c>
-      <c r="B25" s="140" t="s">
+      <c r="B25" s="138" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A26" s="136">
+        <v>45831</v>
+      </c>
+      <c r="B26" s="138" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A27" s="136">
+        <v>45838</v>
+      </c>
+      <c r="B27" s="138" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A28" s="136">
+        <v>45858</v>
+      </c>
+      <c r="B28" s="138" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A29" s="136">
+        <v>45876</v>
+      </c>
+      <c r="B29" s="138" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A30" s="136">
+        <v>45887</v>
+      </c>
+      <c r="B30" s="138" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A31" s="136">
+        <v>45943</v>
+      </c>
+      <c r="B31" s="138" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A32" s="136">
+        <v>45964</v>
+      </c>
+      <c r="B32" s="138" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A33" s="136">
+        <v>45978</v>
+      </c>
+      <c r="B33" s="138" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A34" s="136">
+        <v>45999</v>
+      </c>
+      <c r="B34" s="138" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A35" s="136">
+        <v>46016</v>
+      </c>
+      <c r="B35" s="138" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A36" s="136">
+        <v>46023</v>
+      </c>
+      <c r="B36" s="138" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A26" s="138">
-        <v>45831</v>
-      </c>
-      <c r="B26" s="140" t="s">
+    <row r="37" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A37" s="136">
+        <v>46034</v>
+      </c>
+      <c r="B37" s="138" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A27" s="138">
-        <v>45838</v>
-      </c>
-      <c r="B27" s="140" t="s">
+    <row r="38" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A38" s="136">
+        <v>46104</v>
+      </c>
+      <c r="B38" s="138" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A28" s="138">
-        <v>45858</v>
-      </c>
-      <c r="B28" s="140" t="s">
+    <row r="39" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A39" s="136">
+        <v>46114</v>
+      </c>
+      <c r="B39" s="138" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A29" s="138">
-        <v>45876</v>
-      </c>
-      <c r="B29" s="140" t="s">
+    <row r="40" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A40" s="136">
+        <v>46115</v>
+      </c>
+      <c r="B40" s="138" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A30" s="138">
-        <v>45887</v>
-      </c>
-      <c r="B30" s="140" t="s">
+    <row r="41" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A41" s="136">
+        <v>46143</v>
+      </c>
+      <c r="B41" s="138" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A31" s="138">
-        <v>45943</v>
-      </c>
-      <c r="B31" s="140" t="s">
+    <row r="42" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A42" s="136">
+        <v>46160</v>
+      </c>
+      <c r="B42" s="138" t="s">
         <v>370</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A32" s="138">
-        <v>45964</v>
-      </c>
-      <c r="B32" s="140" t="s">
+    <row r="43" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A43" s="136">
+        <v>46181</v>
+      </c>
+      <c r="B43" s="138" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A33" s="138">
-        <v>45978</v>
-      </c>
-      <c r="B33" s="140" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A34" s="138">
-        <v>45999</v>
-      </c>
-      <c r="B34" s="140" t="s">
+    <row r="44" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A44" s="136">
+        <v>46188</v>
+      </c>
+      <c r="B44" s="138" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A45" s="136">
+        <v>46202</v>
+      </c>
+      <c r="B45" s="138" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A46" s="136">
+        <v>46223</v>
+      </c>
+      <c r="B46" s="138" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A35" s="138">
-        <v>46016</v>
-      </c>
-      <c r="B35" s="140" t="s">
+    <row r="47" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A47" s="136">
+        <v>46241</v>
+      </c>
+      <c r="B47" s="138" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A36" s="138">
-        <v>46023</v>
-      </c>
-      <c r="B36" s="140" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A37" s="138">
-        <v>46034</v>
-      </c>
-      <c r="B37" s="140" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A38" s="138">
-        <v>46104</v>
-      </c>
-      <c r="B38" s="140" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A39" s="138">
-        <v>46114</v>
-      </c>
-      <c r="B39" s="140" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A40" s="138">
-        <v>46115</v>
-      </c>
-      <c r="B40" s="140" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A41" s="138">
-        <v>46143</v>
-      </c>
-      <c r="B41" s="140" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A42" s="138">
-        <v>46160</v>
-      </c>
-      <c r="B42" s="140" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A43" s="138">
-        <v>46181</v>
-      </c>
-      <c r="B43" s="140" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A44" s="138">
-        <v>46188</v>
-      </c>
-      <c r="B44" s="140" t="s">
+    <row r="48" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A48" s="136">
+        <v>46251</v>
+      </c>
+      <c r="B48" s="138" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A45" s="138">
-        <v>46202</v>
-      </c>
-      <c r="B45" s="140" t="s">
+    <row r="49" spans="1:2" ht="17.25" customHeight="1">
+      <c r="A49" s="136">
+        <v>46307</v>
+      </c>
+      <c r="B49" s="138" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A46" s="138">
-        <v>46223</v>
-      </c>
-      <c r="B46" s="140" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A47" s="138">
-        <v>46241</v>
-      </c>
-      <c r="B47" s="140" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A48" s="138">
-        <v>46251</v>
-      </c>
-      <c r="B48" s="140" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A49" s="138">
-        <v>46307</v>
-      </c>
-      <c r="B49" s="140" t="s">
-        <v>370</v>
-      </c>
-    </row>
     <row r="50" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A50" s="138">
+      <c r="A50" s="136">
         <v>46328</v>
       </c>
-      <c r="B50" s="140" t="s">
-        <v>371</v>
+      <c r="B50" s="138" t="s">
+        <v>377</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A51" s="138">
+      <c r="A51" s="136">
         <v>46342</v>
       </c>
-      <c r="B51" s="140" t="s">
-        <v>372</v>
+      <c r="B51" s="138" t="s">
+        <v>378</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A52" s="138">
+      <c r="A52" s="136">
         <v>46364</v>
       </c>
-      <c r="B52" s="140" t="s">
-        <v>373</v>
+      <c r="B52" s="138" t="s">
+        <v>379</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A53" s="138">
+      <c r="A53" s="136">
         <v>46381</v>
       </c>
-      <c r="B53" s="140" t="s">
-        <v>374</v>
+      <c r="B53" s="138" t="s">
+        <v>380</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="17.25" customHeight="1"/>

</xml_diff>

<commit_message>
Actualización de archivos JSON y scripts 09 de Junio 2026
</commit_message>
<xml_diff>
--- a/Tuya.xlsx
+++ b/Tuya.xlsx
@@ -16,19 +16,19 @@
     <sheet name="Hoja2" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'EN PROCESO (Tuya)'!$A$1:$AN$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'EN PROCESO (Tuya)'!$A$1:$AN$136</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="IlaBVRTSKuDodrj1mxssfvkpiQ+B0xnoxgmGJsLK+xo="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="zaziqgNpoVISsllI4B+nz/7Oc9tHu2W8ZCHJjQ2RP7c="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1002" uniqueCount="484">
   <si>
     <t>Asignado a</t>
   </si>
@@ -1205,14 +1205,339 @@
     <t>364</t>
   </si>
   <si>
+    <t>Plan de Continuidad</t>
+  </si>
+  <si>
+    <t>Se requiere realizar el proceso de pruebas del plan de continuidad con el cliente, por lo cual se estara trabajando en contingencia por 24 horas</t>
+  </si>
+  <si>
+    <t>16/03/2026: Cliente se comunica para validar disponibilidad para agendamiento de proceso contingencia, se esta a la espera del email por parte de ellos
+17/03/2026: Notifican agendamiento prueba de continuidad para el 24/03/2026
+24/03/2026: Se realiza el proceso de activacion de plan de continuidad, de acuerdo a lo planeado.
+25/03/2026: Se revierte el plan de continuidad debido a incidente con el aplicativo en el visor de Imagenes por lo que se cancela la prueba y se vuelve al ambiente productivo a las 10am</t>
+  </si>
+  <si>
+    <t>365</t>
+  </si>
+  <si>
     <t>Validación con cliente</t>
   </si>
   <si>
-    <t>Agendamiento para contingencia</t>
-  </si>
-  <si>
-    <t>16/03/2026: Cliente se comunica para validar disponibilidad para agendamiento de proceso contingencia, se esta a la espera del email por parte de ellos
-17/03/2026: Notifican agendamiento prueba de continuidad para el 24/03/2026</t>
+    <t>Se atiende llamada de usuario para validar proceso de unos permisos que requería para unas consultas</t>
+  </si>
+  <si>
+    <t>19/03/2026: Se realizó consulta vía telefónica con el usuario para aclarar dudas que tenía de permisos en aplicativo</t>
+  </si>
+  <si>
+    <t>366</t>
+  </si>
+  <si>
+    <t>Solicitud soportes y bases de morosos a corte 25 Marzo</t>
+  </si>
+  <si>
+    <t>Se genera reporte y se envía información al usuario</t>
+  </si>
+  <si>
+    <t>367</t>
+  </si>
+  <si>
+    <t>Se realiza la validación del caso y se da solución al usuario.</t>
+  </si>
+  <si>
+    <t>368</t>
+  </si>
+  <si>
+    <t>31/03/2026: Se realiza la validación del caso y se da solución al usuario.</t>
+  </si>
+  <si>
+    <t>369</t>
+  </si>
+  <si>
+    <t>Gestión Usuario red</t>
+  </si>
+  <si>
+    <t>Se solicita desbloqueo usuario red</t>
+  </si>
+  <si>
+    <t>30/03/2026: Se realiza solicitud con el cliente para desbloqueo de usuario de red
+31/03/2026: se realiza validación con usuario afectado y se avanza en gestión con el cliente para desbloqueo. se logra desbloqueo de usuario de red</t>
+  </si>
+  <si>
+    <t>370</t>
+  </si>
+  <si>
+    <t>Se realiza la validación de casos y se da solución al usuario.</t>
+  </si>
+  <si>
+    <t>371</t>
+  </si>
+  <si>
+    <t>372</t>
+  </si>
+  <si>
+    <t>Validación Permisos</t>
+  </si>
+  <si>
+    <t>Se realiza validación y actualización de permisos para enviar al cliente y gestionar activación de usuario red</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se realiza solicitud de creación de permisos para usuario de red
+Queda solucionado permisos para el usuario </t>
+  </si>
+  <si>
+    <t>373</t>
+  </si>
+  <si>
+    <t>Evaluación de Riesgos de Proveedores</t>
+  </si>
+  <si>
+    <t>Se requiere diligenciamiento de archivo para evaluación riesgo proveedores</t>
+  </si>
+  <si>
+    <t>EN PROCESO</t>
+  </si>
+  <si>
+    <t>07/04/2026: Se recibe solicitud por parte del cliente para realizar Evalluación de Riesgos proveedores; se esta revisando la información para entrega posterior al cliente
+16/0472026: Se realiza envío de documentación para validación por parte del cliente. Quedamos a la espera de aprobación y confirmación de agendamiento para reunión el 30 de abril de 2026
+17/0472026: El cliente realiza agendamiento de reunión para el 30/04/2026
+30/04/2026: Se presento la evaluación de proveedores sin novedades, se reciben pendientes para enviarles
+04/05/2026: se envían pendientes al cliente, quedamos a la espera de la retroalimentación</t>
+  </si>
+  <si>
+    <t>374</t>
+  </si>
+  <si>
+    <t>Se solicito un informe para saber los clientes que no se tiene soportes</t>
+  </si>
+  <si>
+    <t>10/04/2026: Se genera el reporte y se entrega al area encargada.</t>
+  </si>
+  <si>
+    <t>Natalia y Danilo</t>
+  </si>
+  <si>
+    <t>375</t>
+  </si>
+  <si>
+    <t>Validación Información</t>
+  </si>
+  <si>
+    <t>Usuario solicita información de familias</t>
+  </si>
+  <si>
+    <t>Se realiza validación de información y se comparte al usuario solicitante</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>376</t>
+  </si>
+  <si>
+    <t>Solicitud soportes y bases de morosos a corte 22 de abril</t>
+  </si>
+  <si>
+    <t>Solicitud de usuario para generar base de morosos</t>
+  </si>
+  <si>
+    <t>Usuario envía email solicitando la generación del reporte
+24/04/2026: se genera informe y se realiza el envio al usuario solicitante</t>
+  </si>
+  <si>
+    <t>377</t>
+  </si>
+  <si>
+    <t>Usuario solicita información de familias y permisos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24/04/2026:Se realiza reunión con el cliente para aclarar dudas sobre permisos para gestionar familias </t>
+  </si>
+  <si>
+    <t>378</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cliente radican casos en plataforma </t>
+  </si>
+  <si>
+    <t>04/05/2026: Se realiza la validación del caso, se valida con el area del cliente involucrada en el caso y se da solución al usuario.</t>
+  </si>
+  <si>
+    <t>Faver, Natalia y Danilo</t>
+  </si>
+  <si>
+    <t>379</t>
+  </si>
+  <si>
+    <t>Evaluacion de proveedores</t>
+  </si>
+  <si>
+    <t>Se solicita presentar la evaluacion de proveedores</t>
+  </si>
+  <si>
+    <t>30/04/2026: Se realiza visita a las instalaciones del cliente y se presenta las evaluaciones correspondientes en todo el transcurso del día.</t>
+  </si>
+  <si>
+    <t>380</t>
+  </si>
+  <si>
+    <t>Ejecutar Prueba de Continuidad</t>
+  </si>
+  <si>
+    <t>Se requiere repetira la prueba de continuidad, ya que la prueba anterior no fue satisfactoria y se tuvo que realizar un rollback</t>
+  </si>
+  <si>
+    <t>04/05/2026: Se tiene reunion con el área tecnica del cliente y se programa la prueba para el 11 de Mayo hasta el 12 de Mayo de 2026 
+11/05/2026: Se realiza el proceso de PLan continuidad se ejecutó en la noche el paso y tuvo exito,
+12/05/2026: se trabaja todo el día en contingencia sin errores reporados por el usuario. el día de hoy en la noche se finaliza la prueba de continuidad
+Se finailizo el proceso de continuidad sin errores</t>
+  </si>
+  <si>
+    <t>381</t>
+  </si>
+  <si>
+    <t>Reporte hojas de vida en aplicativo</t>
+  </si>
+  <si>
+    <t>Usuario realiza consulta de cómo se puede gestionar la extracción de información de hojas de vida del aplicativo  nuestro para uno de ellos</t>
+  </si>
+  <si>
+    <t>08/05/2026: Se tiene reunion con el cliente, área implicada de la solicitud (nomina) donde nos indican que requieren la entrega de la hojas de vida que quedaron en el sistema nuestro 
+11/05/2026: agendan reunión con áreas implicadas para validar cómo sería el proceso de generación y entrega de la información
+11/0572026: se tiene nuevamente reunión con el cliente para validación de autorizaciones para generar y enviar la información, se realizara prueba con un documento. El cliente envía email con autorizaicón para gestion y a la espera de respuesta de si se reciben los ddocumentos correctamente
+12/0572026: Se realizo el envío de la información al usuario.
+27/05/2026: Se recibe base para consultar Hv para determinar el tamaño del paquete de datos a transferir
+29/05/2026: Se genera el reporte y se envia la información de los documentos y su peso de todos los documentos.</t>
+  </si>
+  <si>
+    <t>Danilo</t>
+  </si>
+  <si>
+    <t>382</t>
+  </si>
+  <si>
+    <t>Reporte por cliente file sysstema llenos en Imagine</t>
+  </si>
+  <si>
+    <t>Cliente reporta alerta de almacenamiento</t>
+  </si>
+  <si>
+    <t>11/05/2026: Se recibe email por parte del cliente donde nos reportan alertas de almacenamiento en servidor
+se realiza validación y se liberó espacio en los dos discos, se dio respuesta al cliente</t>
+  </si>
+  <si>
+    <t>383</t>
+  </si>
+  <si>
+    <t>12/05/2026: Se valida y se da respuesta al usuario a caso reportado</t>
+  </si>
+  <si>
+    <t>384</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solicitud soporte base moroso </t>
+  </si>
+  <si>
+    <t>Cliente envía solicitud de archivos para un documento en especifico</t>
+  </si>
+  <si>
+    <t>12/05/2026: Se realiza envío de información a la usuaria solicitante</t>
+  </si>
+  <si>
+    <t>385</t>
+  </si>
+  <si>
+    <t>Reporte Alerta Disco</t>
+  </si>
+  <si>
+    <t>Reportan discos llenos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reportan alera por discos llenos, se realiza validacion y se eliminan </t>
+  </si>
+  <si>
+    <t>386</t>
+  </si>
+  <si>
+    <t>Solicitud información usuarios</t>
+  </si>
+  <si>
+    <t>Usuario solicita información de usuarios en ciertas opciones del aplicativo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14/05/2026: Usuario envia email con usuarios para validar si han realizado operaciones en el aplicativo
+20/05/2026: Se esta realizando la validación de la información para enviar al usuario
+20/05/2026: Se realiza la validación de los usuarios, no se encuentran datos y se envia respuesta al usuario solicitante </t>
+  </si>
+  <si>
+    <t>387</t>
+  </si>
+  <si>
+    <t>20/05/2026: Usuario envía email solicitando información
+27/05/2026: Se genera el reporte de los documentos solicitados para planear venta de cartera, se envia inforamción al usuario solicitante.</t>
+  </si>
+  <si>
+    <t>388</t>
+  </si>
+  <si>
+    <t>24//05/2026: Se valida caso asigndo y se da solución requerida</t>
+  </si>
+  <si>
+    <t>389</t>
+  </si>
+  <si>
+    <t>Cliente envía solicitud de archivos para un documento en especifico a 25 de mayo</t>
+  </si>
+  <si>
+    <t>26/05/2026: Cliente envia email con solicitud morosos
+29/05/2026: Se genera reprote con los archivos solicitados y se entrega información al cliente</t>
+  </si>
+  <si>
+    <t>390</t>
+  </si>
+  <si>
+    <t>27//05/2026: Se valida caso asigndo y se da solución requerida</t>
+  </si>
+  <si>
+    <t>391</t>
+  </si>
+  <si>
+    <t>Reunión implementación</t>
+  </si>
+  <si>
+    <t>Reunión Iniciativa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">usuario cita para validacion iniciativa </t>
+  </si>
+  <si>
+    <t>392</t>
+  </si>
+  <si>
+    <t>02/0672026: se realiza validación de casos asigndos, se contacta a usuarios que realizan repore y se da solución requerida</t>
+  </si>
+  <si>
+    <t>393</t>
+  </si>
+  <si>
+    <t>Revision Alertas Almacenamiento</t>
+  </si>
+  <si>
+    <t>Se requiere revision volumenes de almacenamiento</t>
+  </si>
+  <si>
+    <t>04/06/2026: Se realiza revision de los volumenes de almacenamiento.</t>
+  </si>
+  <si>
+    <t>394</t>
+  </si>
+  <si>
+    <t>Solicitud Revision Permisos Usuario</t>
+  </si>
+  <si>
+    <t>Desde seguridad solicitan entregar un informe de uso de pemrisos en el aplicativo de Imagine sobre varios usuarios</t>
+  </si>
+  <si>
+    <t>04/06/2026: Se realiza reunion con los usuarios para aclarar el alcance de la solicitud</t>
   </si>
   <si>
     <t xml:space="preserve"> Año Nuevo</t>
@@ -1330,8 +1655,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd&quot;/&quot;mm&quot;/&quot;yyyy"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="39">
     <font>
@@ -1765,7 +2091,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="139">
+  <cellXfs count="141">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2156,6 +2482,12 @@
     <xf numFmtId="0" fontId="12" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -2388,12 +2720,12 @@
   <sheetPr>
     <tabColor rgb="FF93C47D"/>
   </sheetPr>
-  <dimension ref="A1:AN106"/>
+  <dimension ref="A1:AN136"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.21875" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="10.6640625" customWidth="1"/>
-    <col min="3" max="3" width="24.109375" customWidth="1"/>
+    <col min="3" max="3" width="26.44140625" customWidth="1"/>
     <col min="4" max="4" width="40.33203125" customWidth="1"/>
     <col min="5" max="5" width="19.5546875" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="13.33203125" customWidth="1"/>
@@ -2527,7 +2859,7 @@
       NETWORKDAYS(J2,L2,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>292</v>
+        <v>345</v>
       </c>
       <c r="N2" s="21"/>
       <c r="O2" s="21"/>
@@ -2596,7 +2928,7 @@
       NETWORKDAYS(J3,L3,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>292</v>
+        <v>345</v>
       </c>
       <c r="N3" s="34"/>
       <c r="O3" s="34"/>
@@ -2667,7 +2999,7 @@
       NETWORKDAYS(J4,L4,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>292</v>
+        <v>345</v>
       </c>
       <c r="N4" s="22"/>
       <c r="O4" s="22"/>
@@ -2738,7 +3070,7 @@
       NETWORKDAYS(J5,L5,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>292</v>
+        <v>345</v>
       </c>
       <c r="N5" s="34"/>
       <c r="O5" s="34"/>
@@ -2809,7 +3141,7 @@
       NETWORKDAYS(J6,L6,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>292</v>
+        <v>345</v>
       </c>
       <c r="N6" s="21"/>
       <c r="O6" s="21"/>
@@ -2880,7 +3212,7 @@
       NETWORKDAYS(J7,L7,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>292</v>
+        <v>345</v>
       </c>
       <c r="N7" s="41"/>
       <c r="O7" s="41"/>
@@ -2951,7 +3283,7 @@
       NETWORKDAYS(J8,L8,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>292</v>
+        <v>345</v>
       </c>
       <c r="N8" s="22"/>
       <c r="O8" s="22"/>
@@ -3612,7 +3944,7 @@
       NETWORKDAYS(J17,L17,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>182</v>
+        <v>235</v>
       </c>
       <c r="N17" s="35"/>
       <c r="O17" s="35"/>
@@ -4236,7 +4568,7 @@
       <c r="AM25" s="39"/>
       <c r="AN25" s="39"/>
     </row>
-    <row r="26" spans="1:40" ht="63.75">
+    <row r="26" spans="1:40" ht="51">
       <c r="A26" s="14" t="s">
         <v>18</v>
       </c>
@@ -4924,7 +5256,7 @@
       NETWORKDAYS(J35,L35,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>115</v>
+        <v>168</v>
       </c>
       <c r="N35" s="76"/>
       <c r="O35" s="76">
@@ -5039,7 +5371,7 @@
       <c r="AM36" s="26"/>
       <c r="AN36" s="26"/>
     </row>
-    <row r="37" spans="1:40" ht="25.5">
+    <row r="37" spans="1:40">
       <c r="A37" s="27" t="s">
         <v>18</v>
       </c>
@@ -5183,7 +5515,7 @@
       <c r="AM38" s="26"/>
       <c r="AN38" s="26"/>
     </row>
-    <row r="39" spans="1:40" ht="25.5">
+    <row r="39" spans="1:40">
       <c r="A39" s="27" t="s">
         <v>18</v>
       </c>
@@ -5254,7 +5586,7 @@
       <c r="AM39" s="107"/>
       <c r="AN39" s="108"/>
     </row>
-    <row r="40" spans="1:40" ht="25.5">
+    <row r="40" spans="1:40">
       <c r="A40" s="14" t="s">
         <v>18</v>
       </c>
@@ -5510,7 +5842,7 @@
       NETWORKDAYS(J43,L43,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>113</v>
+        <v>166</v>
       </c>
       <c r="N43" s="41"/>
       <c r="O43" s="41"/>
@@ -9764,7 +10096,7 @@
       <c r="B101" s="130" t="s">
         <v>323</v>
       </c>
-      <c r="C101" s="131" t="s">
+      <c r="C101" s="84" t="s">
         <v>324</v>
       </c>
       <c r="D101" s="90" t="s">
@@ -9803,7 +10135,7 @@
       <c r="N101" s="41"/>
       <c r="O101" s="41"/>
       <c r="P101" s="41"/>
-      <c r="Q101" s="132" t="s">
+      <c r="Q101" s="92" t="s">
         <v>326</v>
       </c>
       <c r="R101" s="133" t="s">
@@ -9839,7 +10171,7 @@
       <c r="B102" s="134" t="s">
         <v>327</v>
       </c>
-      <c r="C102" s="127" t="s">
+      <c r="C102" s="87" t="s">
         <v>328</v>
       </c>
       <c r="D102" s="91" t="s">
@@ -9884,7 +10216,7 @@
       <c r="P102" s="68">
         <v>46087</v>
       </c>
-      <c r="Q102" s="128" t="s">
+      <c r="Q102" s="55" t="s">
         <v>330</v>
       </c>
       <c r="R102" s="129" t="s">
@@ -9913,7 +10245,7 @@
       <c r="AM102" s="118"/>
       <c r="AN102" s="119"/>
     </row>
-    <row r="103" spans="1:40">
+    <row r="103" spans="1:40" ht="48">
       <c r="A103" s="112" t="s">
         <v>331</v>
       </c>
@@ -9961,7 +10293,7 @@
       <c r="N103" s="41"/>
       <c r="O103" s="41"/>
       <c r="P103" s="41"/>
-      <c r="Q103" s="132" t="s">
+      <c r="Q103" s="92" t="s">
         <v>335</v>
       </c>
       <c r="R103" s="133" t="s">
@@ -9997,7 +10329,7 @@
       <c r="B104" s="134" t="s">
         <v>336</v>
       </c>
-      <c r="C104" s="127" t="s">
+      <c r="C104" s="87" t="s">
         <v>337</v>
       </c>
       <c r="D104" s="91" t="s">
@@ -10036,7 +10368,7 @@
       <c r="N104" s="44"/>
       <c r="O104" s="44"/>
       <c r="P104" s="44"/>
-      <c r="Q104" s="128" t="s">
+      <c r="Q104" s="55" t="s">
         <v>339</v>
       </c>
       <c r="R104" s="129" t="s">
@@ -10142,7 +10474,7 @@
       <c r="AM105" s="114"/>
       <c r="AN105" s="115"/>
     </row>
-    <row r="106" spans="1:40">
+    <row r="106" spans="1:40" ht="96">
       <c r="A106" s="116" t="s">
         <v>287</v>
       </c>
@@ -10157,14 +10489,14 @@
       </c>
       <c r="E106" s="93"/>
       <c r="F106" s="103" t="s">
-        <v>251</v>
+        <v>46</v>
       </c>
       <c r="G106" s="104">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H106" s="20">
         <f>IF(OR(J106="",K106="",K106&lt;J106),0,NETWORKDAYS(J106,K106,Hoja2!$A$2:$A$53))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I106" s="68">
         <v>46097</v>
@@ -10172,8 +10504,12 @@
       <c r="J106" s="68">
         <v>46105</v>
       </c>
-      <c r="K106" s="68"/>
-      <c r="L106" s="68"/>
+      <c r="K106" s="68">
+        <v>46106</v>
+      </c>
+      <c r="L106" s="68">
+        <v>46106</v>
+      </c>
       <c r="M106" s="23">
         <f ca="1">IF(OR(J106="",AND(L106="",TODAY()&lt;J106),AND(L106&lt;&gt;"",L106&lt;J106)),0,
    IF(L106="",
@@ -10181,12 +10517,16 @@
       NETWORKDAYS(J106,L106,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>0</v>
-      </c>
-      <c r="N106" s="44"/>
+        <v>2</v>
+      </c>
+      <c r="N106" s="68">
+        <v>46105</v>
+      </c>
       <c r="O106" s="44"/>
-      <c r="P106" s="44"/>
-      <c r="Q106" s="128" t="s">
+      <c r="P106" s="68">
+        <v>46106</v>
+      </c>
+      <c r="Q106" s="55" t="s">
         <v>345</v>
       </c>
       <c r="R106" s="129" t="s">
@@ -10215,18 +10555,2280 @@
       <c r="AM106" s="118"/>
       <c r="AN106" s="119"/>
     </row>
+    <row r="107" spans="1:40" ht="25.5">
+      <c r="A107" s="112" t="s">
+        <v>25</v>
+      </c>
+      <c r="B107" s="130" t="s">
+        <v>346</v>
+      </c>
+      <c r="C107" s="84" t="s">
+        <v>347</v>
+      </c>
+      <c r="D107" s="90" t="s">
+        <v>348</v>
+      </c>
+      <c r="E107" s="95"/>
+      <c r="F107" s="101" t="s">
+        <v>46</v>
+      </c>
+      <c r="G107" s="102">
+        <v>100</v>
+      </c>
+      <c r="H107" s="33">
+        <f>IF(OR(J107="",K107="",K107&lt;J107),0,NETWORKDAYS(J107,K107,Hoja2!$A$2:$A$53))</f>
+        <v>1</v>
+      </c>
+      <c r="I107" s="76">
+        <v>46100</v>
+      </c>
+      <c r="J107" s="76">
+        <v>46100</v>
+      </c>
+      <c r="K107" s="76">
+        <v>46100</v>
+      </c>
+      <c r="L107" s="41"/>
+      <c r="M107" s="36">
+        <f ca="1">IF(OR(J107="",AND(L107="",TODAY()&lt;J107),AND(L107&lt;&gt;"",L107&lt;J107)),0,
+   IF(L107="",
+      NETWORKDAYS(J107,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J107,L107,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>52</v>
+      </c>
+      <c r="N107" s="41"/>
+      <c r="O107" s="41"/>
+      <c r="P107" s="41"/>
+      <c r="Q107" s="92" t="s">
+        <v>349</v>
+      </c>
+      <c r="R107" s="133" t="s">
+        <v>39</v>
+      </c>
+      <c r="S107" s="106"/>
+      <c r="T107" s="107"/>
+      <c r="U107" s="107"/>
+      <c r="V107" s="107"/>
+      <c r="W107" s="107"/>
+      <c r="X107" s="107"/>
+      <c r="Y107" s="107"/>
+      <c r="Z107" s="107"/>
+      <c r="AA107" s="107"/>
+      <c r="AB107" s="107"/>
+      <c r="AC107" s="107"/>
+      <c r="AD107" s="107"/>
+      <c r="AE107" s="107"/>
+      <c r="AF107" s="107"/>
+      <c r="AG107" s="107"/>
+      <c r="AH107" s="107"/>
+      <c r="AI107" s="107"/>
+      <c r="AJ107" s="107"/>
+      <c r="AK107" s="107"/>
+      <c r="AL107" s="107"/>
+      <c r="AM107" s="107"/>
+      <c r="AN107" s="108"/>
+    </row>
+    <row r="108" spans="1:40" ht="38.25">
+      <c r="A108" s="116" t="s">
+        <v>18</v>
+      </c>
+      <c r="B108" s="134" t="s">
+        <v>350</v>
+      </c>
+      <c r="C108" s="87" t="s">
+        <v>351</v>
+      </c>
+      <c r="D108" s="91" t="s">
+        <v>111</v>
+      </c>
+      <c r="E108" s="93"/>
+      <c r="F108" s="103" t="s">
+        <v>46</v>
+      </c>
+      <c r="G108" s="104">
+        <v>0</v>
+      </c>
+      <c r="H108" s="20">
+        <f>IF(OR(J108="",K108="",K108&lt;J108),0,NETWORKDAYS(J108,K108,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I108" s="68">
+        <v>46106</v>
+      </c>
+      <c r="J108" s="44"/>
+      <c r="K108" s="68">
+        <v>46108</v>
+      </c>
+      <c r="L108" s="136">
+        <v>46111</v>
+      </c>
+      <c r="M108" s="23">
+        <f ca="1">IF(OR(J108="",AND(L108="",TODAY()&lt;J108),AND(L108&lt;&gt;"",L108&lt;J108)),0,
+   IF(L108="",
+      NETWORKDAYS(J108,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J108,L108,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
+      </c>
+      <c r="N108" s="44"/>
+      <c r="O108" s="44"/>
+      <c r="P108" s="44"/>
+      <c r="Q108" s="128" t="s">
+        <v>352</v>
+      </c>
+      <c r="R108" s="129" t="s">
+        <v>39</v>
+      </c>
+      <c r="S108" s="117"/>
+      <c r="T108" s="118"/>
+      <c r="U108" s="118"/>
+      <c r="V108" s="118"/>
+      <c r="W108" s="118"/>
+      <c r="X108" s="118"/>
+      <c r="Y108" s="118"/>
+      <c r="Z108" s="118"/>
+      <c r="AA108" s="118"/>
+      <c r="AB108" s="118"/>
+      <c r="AC108" s="118"/>
+      <c r="AD108" s="118"/>
+      <c r="AE108" s="118"/>
+      <c r="AF108" s="118"/>
+      <c r="AG108" s="118"/>
+      <c r="AH108" s="118"/>
+      <c r="AI108" s="118"/>
+      <c r="AJ108" s="118"/>
+      <c r="AK108" s="118"/>
+      <c r="AL108" s="118"/>
+      <c r="AM108" s="118"/>
+      <c r="AN108" s="119"/>
+    </row>
+    <row r="109" spans="1:40">
+      <c r="A109" s="112" t="s">
+        <v>25</v>
+      </c>
+      <c r="B109" s="130" t="s">
+        <v>353</v>
+      </c>
+      <c r="C109" s="84" t="s">
+        <v>204</v>
+      </c>
+      <c r="D109" s="90" t="s">
+        <v>211</v>
+      </c>
+      <c r="E109" s="95"/>
+      <c r="F109" s="101" t="s">
+        <v>46</v>
+      </c>
+      <c r="G109" s="102">
+        <v>100</v>
+      </c>
+      <c r="H109" s="33">
+        <f>IF(OR(J109="",K109="",K109&lt;J109),0,NETWORKDAYS(J109,K109,Hoja2!$A$2:$A$53))</f>
+        <v>1</v>
+      </c>
+      <c r="I109" s="76">
+        <v>46108</v>
+      </c>
+      <c r="J109" s="76">
+        <v>46108</v>
+      </c>
+      <c r="K109" s="76">
+        <v>46108</v>
+      </c>
+      <c r="L109" s="76">
+        <v>46108</v>
+      </c>
+      <c r="M109" s="36">
+        <f ca="1">IF(OR(J109="",AND(L109="",TODAY()&lt;J109),AND(L109&lt;&gt;"",L109&lt;J109)),0,
+   IF(L109="",
+      NETWORKDAYS(J109,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J109,L109,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N109" s="41"/>
+      <c r="O109" s="41"/>
+      <c r="P109" s="41"/>
+      <c r="Q109" s="92" t="s">
+        <v>354</v>
+      </c>
+      <c r="R109" s="133" t="s">
+        <v>39</v>
+      </c>
+      <c r="S109" s="113"/>
+      <c r="T109" s="114"/>
+      <c r="U109" s="114"/>
+      <c r="V109" s="114"/>
+      <c r="W109" s="114"/>
+      <c r="X109" s="114"/>
+      <c r="Y109" s="114"/>
+      <c r="Z109" s="114"/>
+      <c r="AA109" s="114"/>
+      <c r="AB109" s="114"/>
+      <c r="AC109" s="114"/>
+      <c r="AD109" s="114"/>
+      <c r="AE109" s="114"/>
+      <c r="AF109" s="114"/>
+      <c r="AG109" s="114"/>
+      <c r="AH109" s="114"/>
+      <c r="AI109" s="114"/>
+      <c r="AJ109" s="114"/>
+      <c r="AK109" s="114"/>
+      <c r="AL109" s="114"/>
+      <c r="AM109" s="114"/>
+      <c r="AN109" s="115"/>
+    </row>
+    <row r="110" spans="1:40">
+      <c r="A110" s="116" t="s">
+        <v>287</v>
+      </c>
+      <c r="B110" s="134" t="s">
+        <v>355</v>
+      </c>
+      <c r="C110" s="87" t="s">
+        <v>204</v>
+      </c>
+      <c r="D110" s="91" t="s">
+        <v>211</v>
+      </c>
+      <c r="E110" s="93"/>
+      <c r="F110" s="103" t="s">
+        <v>46</v>
+      </c>
+      <c r="G110" s="104">
+        <v>100</v>
+      </c>
+      <c r="H110" s="20">
+        <f>IF(OR(J110="",K110="",K110&lt;J110),0,NETWORKDAYS(J110,K110,Hoja2!$A$2:$A$53))</f>
+        <v>1</v>
+      </c>
+      <c r="I110" s="68">
+        <v>46112</v>
+      </c>
+      <c r="J110" s="68">
+        <v>46112</v>
+      </c>
+      <c r="K110" s="68">
+        <v>46112</v>
+      </c>
+      <c r="L110" s="68">
+        <v>46112</v>
+      </c>
+      <c r="M110" s="23">
+        <f ca="1">IF(OR(J110="",AND(L110="",TODAY()&lt;J110),AND(L110&lt;&gt;"",L110&lt;J110)),0,
+   IF(L110="",
+      NETWORKDAYS(J110,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J110,L110,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N110" s="44"/>
+      <c r="O110" s="44"/>
+      <c r="P110" s="44"/>
+      <c r="Q110" s="55" t="s">
+        <v>356</v>
+      </c>
+      <c r="R110" s="129" t="s">
+        <v>39</v>
+      </c>
+      <c r="S110" s="117"/>
+      <c r="T110" s="118"/>
+      <c r="U110" s="118"/>
+      <c r="V110" s="118"/>
+      <c r="W110" s="118"/>
+      <c r="X110" s="118"/>
+      <c r="Y110" s="118"/>
+      <c r="Z110" s="118"/>
+      <c r="AA110" s="118"/>
+      <c r="AB110" s="118"/>
+      <c r="AC110" s="118"/>
+      <c r="AD110" s="118"/>
+      <c r="AE110" s="118"/>
+      <c r="AF110" s="118"/>
+      <c r="AG110" s="118"/>
+      <c r="AH110" s="118"/>
+      <c r="AI110" s="118"/>
+      <c r="AJ110" s="118"/>
+      <c r="AK110" s="118"/>
+      <c r="AL110" s="118"/>
+      <c r="AM110" s="118"/>
+      <c r="AN110" s="119"/>
+    </row>
+    <row r="111" spans="1:40" ht="36">
+      <c r="A111" s="112" t="s">
+        <v>25</v>
+      </c>
+      <c r="B111" s="130" t="s">
+        <v>357</v>
+      </c>
+      <c r="C111" s="84" t="s">
+        <v>358</v>
+      </c>
+      <c r="D111" s="90" t="s">
+        <v>359</v>
+      </c>
+      <c r="E111" s="95"/>
+      <c r="F111" s="101" t="s">
+        <v>46</v>
+      </c>
+      <c r="G111" s="102">
+        <v>100</v>
+      </c>
+      <c r="H111" s="33">
+        <f>IF(OR(J111="",K111="",K111&lt;J111),0,NETWORKDAYS(J111,K111,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I111" s="76">
+        <v>46111</v>
+      </c>
+      <c r="J111" s="76"/>
+      <c r="K111" s="76">
+        <v>46112</v>
+      </c>
+      <c r="L111" s="76">
+        <v>46112</v>
+      </c>
+      <c r="M111" s="36">
+        <f ca="1">IF(OR(J111="",AND(L111="",TODAY()&lt;J111),AND(L111&lt;&gt;"",L111&lt;J111)),0,
+   IF(L111="",
+      NETWORKDAYS(J111,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J111,L111,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
+      </c>
+      <c r="N111" s="41"/>
+      <c r="O111" s="41"/>
+      <c r="P111" s="41"/>
+      <c r="Q111" s="92" t="s">
+        <v>360</v>
+      </c>
+      <c r="R111" s="133" t="s">
+        <v>39</v>
+      </c>
+      <c r="S111" s="113"/>
+      <c r="T111" s="114"/>
+      <c r="U111" s="114"/>
+      <c r="V111" s="114"/>
+      <c r="W111" s="114"/>
+      <c r="X111" s="114"/>
+      <c r="Y111" s="114"/>
+      <c r="Z111" s="114"/>
+      <c r="AA111" s="114"/>
+      <c r="AB111" s="114"/>
+      <c r="AC111" s="114"/>
+      <c r="AD111" s="114"/>
+      <c r="AE111" s="114"/>
+      <c r="AF111" s="114"/>
+      <c r="AG111" s="114"/>
+      <c r="AH111" s="114"/>
+      <c r="AI111" s="114"/>
+      <c r="AJ111" s="114"/>
+      <c r="AK111" s="114"/>
+      <c r="AL111" s="114"/>
+      <c r="AM111" s="114"/>
+      <c r="AN111" s="115"/>
+    </row>
+    <row r="112" spans="1:40">
+      <c r="A112" s="116" t="s">
+        <v>25</v>
+      </c>
+      <c r="B112" s="134" t="s">
+        <v>361</v>
+      </c>
+      <c r="C112" s="87" t="s">
+        <v>204</v>
+      </c>
+      <c r="D112" s="91" t="s">
+        <v>211</v>
+      </c>
+      <c r="E112" s="93"/>
+      <c r="F112" s="103" t="s">
+        <v>46</v>
+      </c>
+      <c r="G112" s="104">
+        <v>100</v>
+      </c>
+      <c r="H112" s="20">
+        <f>IF(OR(J112="",K112="",K112&lt;J112),0,NETWORKDAYS(J112,K112,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I112" s="68">
+        <v>46113</v>
+      </c>
+      <c r="J112" s="68"/>
+      <c r="K112" s="68">
+        <v>46113</v>
+      </c>
+      <c r="L112" s="68">
+        <v>46113</v>
+      </c>
+      <c r="M112" s="23">
+        <f ca="1">IF(OR(J112="",AND(L112="",TODAY()&lt;J112),AND(L112&lt;&gt;"",L112&lt;J112)),0,
+   IF(L112="",
+      NETWORKDAYS(J112,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J112,L112,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
+      </c>
+      <c r="N112" s="44"/>
+      <c r="O112" s="44"/>
+      <c r="P112" s="44"/>
+      <c r="Q112" s="55" t="s">
+        <v>362</v>
+      </c>
+      <c r="R112" s="129" t="s">
+        <v>39</v>
+      </c>
+      <c r="S112" s="117"/>
+      <c r="T112" s="118"/>
+      <c r="U112" s="118"/>
+      <c r="V112" s="118"/>
+      <c r="W112" s="118"/>
+      <c r="X112" s="118"/>
+      <c r="Y112" s="118"/>
+      <c r="Z112" s="118"/>
+      <c r="AA112" s="118"/>
+      <c r="AB112" s="118"/>
+      <c r="AC112" s="118"/>
+      <c r="AD112" s="118"/>
+      <c r="AE112" s="118"/>
+      <c r="AF112" s="118"/>
+      <c r="AG112" s="118"/>
+      <c r="AH112" s="118"/>
+      <c r="AI112" s="118"/>
+      <c r="AJ112" s="118"/>
+      <c r="AK112" s="118"/>
+      <c r="AL112" s="118"/>
+      <c r="AM112" s="118"/>
+      <c r="AN112" s="119"/>
+    </row>
+    <row r="113" spans="1:40">
+      <c r="A113" s="112" t="s">
+        <v>25</v>
+      </c>
+      <c r="B113" s="130" t="s">
+        <v>363</v>
+      </c>
+      <c r="C113" s="84" t="s">
+        <v>204</v>
+      </c>
+      <c r="D113" s="90" t="s">
+        <v>211</v>
+      </c>
+      <c r="E113" s="95"/>
+      <c r="F113" s="101" t="s">
+        <v>46</v>
+      </c>
+      <c r="G113" s="102">
+        <v>100</v>
+      </c>
+      <c r="H113" s="33">
+        <f>IF(OR(J113="",K113="",K113&lt;J113),0,NETWORKDAYS(J113,K113,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I113" s="76">
+        <v>46118</v>
+      </c>
+      <c r="J113" s="76"/>
+      <c r="K113" s="76">
+        <v>46118</v>
+      </c>
+      <c r="L113" s="76">
+        <v>46118</v>
+      </c>
+      <c r="M113" s="36">
+        <f ca="1">IF(OR(J113="",AND(L113="",TODAY()&lt;J113),AND(L113&lt;&gt;"",L113&lt;J113)),0,
+   IF(L113="",
+      NETWORKDAYS(J113,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J113,L113,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
+      </c>
+      <c r="N113" s="41"/>
+      <c r="O113" s="41"/>
+      <c r="P113" s="41"/>
+      <c r="Q113" s="92" t="s">
+        <v>362</v>
+      </c>
+      <c r="R113" s="133" t="s">
+        <v>39</v>
+      </c>
+      <c r="S113" s="113"/>
+      <c r="T113" s="114"/>
+      <c r="U113" s="114"/>
+      <c r="V113" s="114"/>
+      <c r="W113" s="114"/>
+      <c r="X113" s="114"/>
+      <c r="Y113" s="114"/>
+      <c r="Z113" s="114"/>
+      <c r="AA113" s="114"/>
+      <c r="AB113" s="114"/>
+      <c r="AC113" s="114"/>
+      <c r="AD113" s="114"/>
+      <c r="AE113" s="114"/>
+      <c r="AF113" s="114"/>
+      <c r="AG113" s="114"/>
+      <c r="AH113" s="114"/>
+      <c r="AI113" s="114"/>
+      <c r="AJ113" s="114"/>
+      <c r="AK113" s="114"/>
+      <c r="AL113" s="114"/>
+      <c r="AM113" s="114"/>
+      <c r="AN113" s="115"/>
+    </row>
+    <row r="114" spans="1:40" ht="25.5">
+      <c r="A114" s="116" t="s">
+        <v>287</v>
+      </c>
+      <c r="B114" s="134" t="s">
+        <v>364</v>
+      </c>
+      <c r="C114" s="87" t="s">
+        <v>365</v>
+      </c>
+      <c r="D114" s="91" t="s">
+        <v>366</v>
+      </c>
+      <c r="E114" s="93"/>
+      <c r="F114" s="103" t="s">
+        <v>46</v>
+      </c>
+      <c r="G114" s="104">
+        <v>100</v>
+      </c>
+      <c r="H114" s="20">
+        <f>IF(OR(J114="",K114="",K114&lt;J114),0,NETWORKDAYS(J114,K114,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I114" s="68">
+        <v>46119</v>
+      </c>
+      <c r="J114" s="68"/>
+      <c r="K114" s="68">
+        <v>46119</v>
+      </c>
+      <c r="L114" s="68">
+        <v>46119</v>
+      </c>
+      <c r="M114" s="23">
+        <f ca="1">IF(OR(J114="",AND(L114="",TODAY()&lt;J114),AND(L114&lt;&gt;"",L114&lt;J114)),0,
+   IF(L114="",
+      NETWORKDAYS(J114,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J114,L114,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
+      </c>
+      <c r="N114" s="44"/>
+      <c r="O114" s="44"/>
+      <c r="P114" s="44"/>
+      <c r="Q114" s="55" t="s">
+        <v>367</v>
+      </c>
+      <c r="R114" s="129" t="s">
+        <v>39</v>
+      </c>
+      <c r="S114" s="117"/>
+      <c r="T114" s="118"/>
+      <c r="U114" s="118"/>
+      <c r="V114" s="118"/>
+      <c r="W114" s="118"/>
+      <c r="X114" s="118"/>
+      <c r="Y114" s="118"/>
+      <c r="Z114" s="118"/>
+      <c r="AA114" s="118"/>
+      <c r="AB114" s="118"/>
+      <c r="AC114" s="118"/>
+      <c r="AD114" s="118"/>
+      <c r="AE114" s="118"/>
+      <c r="AF114" s="118"/>
+      <c r="AG114" s="118"/>
+      <c r="AH114" s="118"/>
+      <c r="AI114" s="118"/>
+      <c r="AJ114" s="118"/>
+      <c r="AK114" s="118"/>
+      <c r="AL114" s="118"/>
+      <c r="AM114" s="118"/>
+      <c r="AN114" s="119"/>
+    </row>
+    <row r="115" spans="1:40" ht="120">
+      <c r="A115" s="112" t="s">
+        <v>25</v>
+      </c>
+      <c r="B115" s="130" t="s">
+        <v>368</v>
+      </c>
+      <c r="C115" s="84" t="s">
+        <v>369</v>
+      </c>
+      <c r="D115" s="90" t="s">
+        <v>370</v>
+      </c>
+      <c r="E115" s="95"/>
+      <c r="F115" s="101" t="s">
+        <v>371</v>
+      </c>
+      <c r="G115" s="102">
+        <v>90</v>
+      </c>
+      <c r="H115" s="33">
+        <f>IF(OR(J115="",K115="",K115&lt;J115),0,NETWORKDAYS(J115,K115,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I115" s="76">
+        <v>46119</v>
+      </c>
+      <c r="J115" s="76"/>
+      <c r="K115" s="76">
+        <v>46135</v>
+      </c>
+      <c r="L115" s="76"/>
+      <c r="M115" s="36">
+        <f ca="1">IF(OR(J115="",AND(L115="",TODAY()&lt;J115),AND(L115&lt;&gt;"",L115&lt;J115)),0,
+   IF(L115="",
+      NETWORKDAYS(J115,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J115,L115,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
+      </c>
+      <c r="N115" s="41"/>
+      <c r="O115" s="41"/>
+      <c r="P115" s="41"/>
+      <c r="Q115" s="92" t="s">
+        <v>372</v>
+      </c>
+      <c r="R115" s="133" t="s">
+        <v>39</v>
+      </c>
+      <c r="S115" s="113"/>
+      <c r="T115" s="114"/>
+      <c r="U115" s="114"/>
+      <c r="V115" s="114"/>
+      <c r="W115" s="114"/>
+      <c r="X115" s="114"/>
+      <c r="Y115" s="114"/>
+      <c r="Z115" s="114"/>
+      <c r="AA115" s="114"/>
+      <c r="AB115" s="114"/>
+      <c r="AC115" s="114"/>
+      <c r="AD115" s="114"/>
+      <c r="AE115" s="114"/>
+      <c r="AF115" s="114"/>
+      <c r="AG115" s="114"/>
+      <c r="AH115" s="114"/>
+      <c r="AI115" s="114"/>
+      <c r="AJ115" s="114"/>
+      <c r="AK115" s="114"/>
+      <c r="AL115" s="114"/>
+      <c r="AM115" s="114"/>
+      <c r="AN115" s="115"/>
+    </row>
+    <row r="116" spans="1:40" ht="25.5">
+      <c r="A116" s="116" t="s">
+        <v>18</v>
+      </c>
+      <c r="B116" s="134" t="s">
+        <v>373</v>
+      </c>
+      <c r="C116" s="87" t="s">
+        <v>315</v>
+      </c>
+      <c r="D116" s="91" t="s">
+        <v>374</v>
+      </c>
+      <c r="E116" s="93"/>
+      <c r="F116" s="103" t="s">
+        <v>46</v>
+      </c>
+      <c r="G116" s="104">
+        <v>100</v>
+      </c>
+      <c r="H116" s="20">
+        <f>IF(OR(J116="",K116="",K116&lt;J116),0,NETWORKDAYS(J116,K116,Hoja2!$A$2:$A$53))</f>
+        <v>1</v>
+      </c>
+      <c r="I116" s="68">
+        <v>46122</v>
+      </c>
+      <c r="J116" s="68">
+        <v>46122</v>
+      </c>
+      <c r="K116" s="68">
+        <v>46122</v>
+      </c>
+      <c r="L116" s="68">
+        <v>46122</v>
+      </c>
+      <c r="M116" s="23">
+        <f ca="1">IF(OR(J116="",AND(L116="",TODAY()&lt;J116),AND(L116&lt;&gt;"",L116&lt;J116)),0,
+   IF(L116="",
+      NETWORKDAYS(J116,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J116,L116,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N116" s="44">
+        <v>46122</v>
+      </c>
+      <c r="O116" s="44"/>
+      <c r="P116" s="44"/>
+      <c r="Q116" s="55" t="s">
+        <v>375</v>
+      </c>
+      <c r="R116" s="129" t="s">
+        <v>39</v>
+      </c>
+      <c r="S116" s="117"/>
+      <c r="T116" s="118"/>
+      <c r="U116" s="118"/>
+      <c r="V116" s="118"/>
+      <c r="W116" s="118"/>
+      <c r="X116" s="118"/>
+      <c r="Y116" s="118"/>
+      <c r="Z116" s="118"/>
+      <c r="AA116" s="118"/>
+      <c r="AB116" s="118"/>
+      <c r="AC116" s="118"/>
+      <c r="AD116" s="118"/>
+      <c r="AE116" s="118"/>
+      <c r="AF116" s="118"/>
+      <c r="AG116" s="118"/>
+      <c r="AH116" s="118"/>
+      <c r="AI116" s="118"/>
+      <c r="AJ116" s="118"/>
+      <c r="AK116" s="118"/>
+      <c r="AL116" s="118"/>
+      <c r="AM116" s="118"/>
+      <c r="AN116" s="119"/>
+    </row>
+    <row r="117" spans="1:40">
+      <c r="A117" s="112" t="s">
+        <v>376</v>
+      </c>
+      <c r="B117" s="130" t="s">
+        <v>377</v>
+      </c>
+      <c r="C117" s="84" t="s">
+        <v>378</v>
+      </c>
+      <c r="D117" s="90" t="s">
+        <v>379</v>
+      </c>
+      <c r="E117" s="95"/>
+      <c r="F117" s="101" t="s">
+        <v>46</v>
+      </c>
+      <c r="G117" s="102">
+        <v>100</v>
+      </c>
+      <c r="H117" s="33">
+        <f>IF(OR(J117="",K117="",K117&lt;J117),0,NETWORKDAYS(J117,K117,Hoja2!$A$2:$A$53))</f>
+        <v>1</v>
+      </c>
+      <c r="I117" s="76">
+        <v>46134</v>
+      </c>
+      <c r="J117" s="76">
+        <v>46134</v>
+      </c>
+      <c r="K117" s="76">
+        <v>46134</v>
+      </c>
+      <c r="L117" s="76">
+        <v>46134</v>
+      </c>
+      <c r="M117" s="36">
+        <f ca="1">IF(OR(J117="",AND(L117="",TODAY()&lt;J117),AND(L117&lt;&gt;"",L117&lt;J117)),0,
+   IF(L117="",
+      NETWORKDAYS(J117,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J117,L117,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N117" s="41"/>
+      <c r="O117" s="41"/>
+      <c r="P117" s="41"/>
+      <c r="Q117" s="92" t="s">
+        <v>380</v>
+      </c>
+      <c r="R117" s="133" t="s">
+        <v>381</v>
+      </c>
+      <c r="S117" s="113"/>
+      <c r="T117" s="114"/>
+      <c r="U117" s="114"/>
+      <c r="V117" s="114"/>
+      <c r="W117" s="114"/>
+      <c r="X117" s="114"/>
+      <c r="Y117" s="114"/>
+      <c r="Z117" s="114"/>
+      <c r="AA117" s="114"/>
+      <c r="AB117" s="114"/>
+      <c r="AC117" s="114"/>
+      <c r="AD117" s="114"/>
+      <c r="AE117" s="114"/>
+      <c r="AF117" s="114"/>
+      <c r="AG117" s="114"/>
+      <c r="AH117" s="114"/>
+      <c r="AI117" s="114"/>
+      <c r="AJ117" s="114"/>
+      <c r="AK117" s="114"/>
+      <c r="AL117" s="114"/>
+      <c r="AM117" s="114"/>
+      <c r="AN117" s="115"/>
+    </row>
+    <row r="118" spans="1:40" ht="25.5">
+      <c r="A118" s="116" t="s">
+        <v>376</v>
+      </c>
+      <c r="B118" s="134" t="s">
+        <v>382</v>
+      </c>
+      <c r="C118" s="87" t="s">
+        <v>383</v>
+      </c>
+      <c r="D118" s="91" t="s">
+        <v>384</v>
+      </c>
+      <c r="E118" s="93"/>
+      <c r="F118" s="103" t="s">
+        <v>46</v>
+      </c>
+      <c r="G118" s="104">
+        <v>100</v>
+      </c>
+      <c r="H118" s="20">
+        <f>IF(OR(J118="",K118="",K118&lt;J118),0,NETWORKDAYS(J118,K118,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I118" s="68">
+        <v>46135</v>
+      </c>
+      <c r="J118" s="68"/>
+      <c r="K118" s="68">
+        <v>46136</v>
+      </c>
+      <c r="L118" s="68">
+        <v>46136</v>
+      </c>
+      <c r="M118" s="23">
+        <f ca="1">IF(OR(J118="",AND(L118="",TODAY()&lt;J118),AND(L118&lt;&gt;"",L118&lt;J118)),0,
+   IF(L118="",
+      NETWORKDAYS(J118,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J118,L118,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
+      </c>
+      <c r="N118" s="44"/>
+      <c r="O118" s="44"/>
+      <c r="P118" s="44"/>
+      <c r="Q118" s="55" t="s">
+        <v>385</v>
+      </c>
+      <c r="R118" s="129" t="s">
+        <v>39</v>
+      </c>
+      <c r="S118" s="117"/>
+      <c r="T118" s="118"/>
+      <c r="U118" s="118"/>
+      <c r="V118" s="118"/>
+      <c r="W118" s="118"/>
+      <c r="X118" s="118"/>
+      <c r="Y118" s="118"/>
+      <c r="Z118" s="118"/>
+      <c r="AA118" s="118"/>
+      <c r="AB118" s="118"/>
+      <c r="AC118" s="118"/>
+      <c r="AD118" s="118"/>
+      <c r="AE118" s="118"/>
+      <c r="AF118" s="118"/>
+      <c r="AG118" s="118"/>
+      <c r="AH118" s="118"/>
+      <c r="AI118" s="118"/>
+      <c r="AJ118" s="118"/>
+      <c r="AK118" s="118"/>
+      <c r="AL118" s="118"/>
+      <c r="AM118" s="118"/>
+      <c r="AN118" s="119"/>
+    </row>
+    <row r="119" spans="1:40" ht="24">
+      <c r="A119" s="112" t="s">
+        <v>25</v>
+      </c>
+      <c r="B119" s="130" t="s">
+        <v>386</v>
+      </c>
+      <c r="C119" s="84" t="s">
+        <v>378</v>
+      </c>
+      <c r="D119" s="90" t="s">
+        <v>387</v>
+      </c>
+      <c r="E119" s="95"/>
+      <c r="F119" s="101" t="s">
+        <v>46</v>
+      </c>
+      <c r="G119" s="102">
+        <v>100</v>
+      </c>
+      <c r="H119" s="33">
+        <f>IF(OR(J119="",K119="",K119&lt;J119),0,NETWORKDAYS(J119,K119,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I119" s="76">
+        <v>46136</v>
+      </c>
+      <c r="J119" s="76">
+        <v>46136</v>
+      </c>
+      <c r="K119" s="76"/>
+      <c r="L119" s="76">
+        <v>46136</v>
+      </c>
+      <c r="M119" s="36">
+        <f ca="1">IF(OR(J119="",AND(L119="",TODAY()&lt;J119),AND(L119&lt;&gt;"",L119&lt;J119)),0,
+   IF(L119="",
+      NETWORKDAYS(J119,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J119,L119,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N119" s="41"/>
+      <c r="O119" s="41"/>
+      <c r="P119" s="41"/>
+      <c r="Q119" s="92" t="s">
+        <v>388</v>
+      </c>
+      <c r="R119" s="133" t="s">
+        <v>381</v>
+      </c>
+      <c r="S119" s="113"/>
+      <c r="T119" s="114"/>
+      <c r="U119" s="114"/>
+      <c r="V119" s="114"/>
+      <c r="W119" s="114"/>
+      <c r="X119" s="114"/>
+      <c r="Y119" s="114"/>
+      <c r="Z119" s="114"/>
+      <c r="AA119" s="114"/>
+      <c r="AB119" s="114"/>
+      <c r="AC119" s="114"/>
+      <c r="AD119" s="114"/>
+      <c r="AE119" s="114"/>
+      <c r="AF119" s="114"/>
+      <c r="AG119" s="114"/>
+      <c r="AH119" s="114"/>
+      <c r="AI119" s="114"/>
+      <c r="AJ119" s="114"/>
+      <c r="AK119" s="114"/>
+      <c r="AL119" s="114"/>
+      <c r="AM119" s="114"/>
+      <c r="AN119" s="115"/>
+    </row>
+    <row r="120" spans="1:40" ht="24">
+      <c r="A120" s="116" t="s">
+        <v>287</v>
+      </c>
+      <c r="B120" s="134" t="s">
+        <v>389</v>
+      </c>
+      <c r="C120" s="87" t="s">
+        <v>204</v>
+      </c>
+      <c r="D120" s="91" t="s">
+        <v>390</v>
+      </c>
+      <c r="E120" s="93"/>
+      <c r="F120" s="103" t="s">
+        <v>46</v>
+      </c>
+      <c r="G120" s="104">
+        <v>100</v>
+      </c>
+      <c r="H120" s="20">
+        <f>IF(OR(J120="",K120="",K120&lt;J120),0,NETWORKDAYS(J120,K120,Hoja2!$A$2:$A$53))</f>
+        <v>1</v>
+      </c>
+      <c r="I120" s="68">
+        <v>46146</v>
+      </c>
+      <c r="J120" s="68">
+        <v>46146</v>
+      </c>
+      <c r="K120" s="68">
+        <v>46146</v>
+      </c>
+      <c r="L120" s="68">
+        <v>46146</v>
+      </c>
+      <c r="M120" s="23">
+        <f ca="1">IF(OR(J120="",AND(L120="",TODAY()&lt;J120),AND(L120&lt;&gt;"",L120&lt;J120)),0,
+   IF(L120="",
+      NETWORKDAYS(J120,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J120,L120,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N120" s="44"/>
+      <c r="O120" s="44"/>
+      <c r="P120" s="44"/>
+      <c r="Q120" s="55" t="s">
+        <v>391</v>
+      </c>
+      <c r="R120" s="129" t="s">
+        <v>39</v>
+      </c>
+      <c r="S120" s="117"/>
+      <c r="T120" s="118"/>
+      <c r="U120" s="118"/>
+      <c r="V120" s="118"/>
+      <c r="W120" s="118"/>
+      <c r="X120" s="118"/>
+      <c r="Y120" s="118"/>
+      <c r="Z120" s="118"/>
+      <c r="AA120" s="118"/>
+      <c r="AB120" s="118"/>
+      <c r="AC120" s="118"/>
+      <c r="AD120" s="118"/>
+      <c r="AE120" s="118"/>
+      <c r="AF120" s="118"/>
+      <c r="AG120" s="118"/>
+      <c r="AH120" s="118"/>
+      <c r="AI120" s="118"/>
+      <c r="AJ120" s="118"/>
+      <c r="AK120" s="118"/>
+      <c r="AL120" s="118"/>
+      <c r="AM120" s="118"/>
+      <c r="AN120" s="119"/>
+    </row>
+    <row r="121" spans="1:40" ht="24">
+      <c r="A121" s="112" t="s">
+        <v>392</v>
+      </c>
+      <c r="B121" s="130" t="s">
+        <v>393</v>
+      </c>
+      <c r="C121" s="84" t="s">
+        <v>394</v>
+      </c>
+      <c r="D121" s="90" t="s">
+        <v>395</v>
+      </c>
+      <c r="E121" s="95"/>
+      <c r="F121" s="101" t="s">
+        <v>46</v>
+      </c>
+      <c r="G121" s="102">
+        <v>100</v>
+      </c>
+      <c r="H121" s="33">
+        <f>IF(OR(J121="",K121="",K121&lt;J121),0,NETWORKDAYS(J121,K121,Hoja2!$A$2:$A$53))</f>
+        <v>1</v>
+      </c>
+      <c r="I121" s="76">
+        <v>46142</v>
+      </c>
+      <c r="J121" s="76">
+        <v>46142</v>
+      </c>
+      <c r="K121" s="76">
+        <v>46142</v>
+      </c>
+      <c r="L121" s="76">
+        <v>46142</v>
+      </c>
+      <c r="M121" s="36">
+        <f ca="1">IF(OR(J121="",AND(L121="",TODAY()&lt;J121),AND(L121&lt;&gt;"",L121&lt;J121)),0,
+   IF(L121="",
+      NETWORKDAYS(J121,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J121,L121,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N121" s="41"/>
+      <c r="O121" s="41"/>
+      <c r="P121" s="41"/>
+      <c r="Q121" s="92" t="s">
+        <v>396</v>
+      </c>
+      <c r="R121" s="133" t="s">
+        <v>39</v>
+      </c>
+      <c r="S121" s="113"/>
+      <c r="T121" s="114"/>
+      <c r="U121" s="114"/>
+      <c r="V121" s="114"/>
+      <c r="W121" s="114"/>
+      <c r="X121" s="114"/>
+      <c r="Y121" s="114"/>
+      <c r="Z121" s="114"/>
+      <c r="AA121" s="114"/>
+      <c r="AB121" s="114"/>
+      <c r="AC121" s="114"/>
+      <c r="AD121" s="114"/>
+      <c r="AE121" s="114"/>
+      <c r="AF121" s="114"/>
+      <c r="AG121" s="114"/>
+      <c r="AH121" s="114"/>
+      <c r="AI121" s="114"/>
+      <c r="AJ121" s="114"/>
+      <c r="AK121" s="114"/>
+      <c r="AL121" s="114"/>
+      <c r="AM121" s="114"/>
+      <c r="AN121" s="115"/>
+    </row>
+    <row r="122" spans="1:40" ht="84">
+      <c r="A122" s="116" t="s">
+        <v>392</v>
+      </c>
+      <c r="B122" s="134" t="s">
+        <v>397</v>
+      </c>
+      <c r="C122" s="87" t="s">
+        <v>398</v>
+      </c>
+      <c r="D122" s="91" t="s">
+        <v>399</v>
+      </c>
+      <c r="E122" s="93"/>
+      <c r="F122" s="103" t="s">
+        <v>46</v>
+      </c>
+      <c r="G122" s="104">
+        <v>50</v>
+      </c>
+      <c r="H122" s="20">
+        <f>IF(OR(J122="",K122="",K122&lt;J122),0,NETWORKDAYS(J122,K122,Hoja2!$A$2:$A$53))</f>
+        <v>2</v>
+      </c>
+      <c r="I122" s="68">
+        <v>46146</v>
+      </c>
+      <c r="J122" s="68">
+        <v>46153</v>
+      </c>
+      <c r="K122" s="68">
+        <v>46154</v>
+      </c>
+      <c r="L122" s="68">
+        <v>46154</v>
+      </c>
+      <c r="M122" s="23">
+        <f ca="1">IF(OR(J122="",AND(L122="",TODAY()&lt;J122),AND(L122&lt;&gt;"",L122&lt;J122)),0,
+   IF(L122="",
+      NETWORKDAYS(J122,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J122,L122,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>2</v>
+      </c>
+      <c r="N122" s="44">
+        <v>46154</v>
+      </c>
+      <c r="O122" s="44"/>
+      <c r="P122" s="44"/>
+      <c r="Q122" s="55" t="s">
+        <v>400</v>
+      </c>
+      <c r="R122" s="129" t="s">
+        <v>39</v>
+      </c>
+      <c r="S122" s="117"/>
+      <c r="T122" s="118"/>
+      <c r="U122" s="118"/>
+      <c r="V122" s="118"/>
+      <c r="W122" s="118"/>
+      <c r="X122" s="118"/>
+      <c r="Y122" s="118"/>
+      <c r="Z122" s="118"/>
+      <c r="AA122" s="118"/>
+      <c r="AB122" s="118"/>
+      <c r="AC122" s="118"/>
+      <c r="AD122" s="118"/>
+      <c r="AE122" s="118"/>
+      <c r="AF122" s="118"/>
+      <c r="AG122" s="118"/>
+      <c r="AH122" s="118"/>
+      <c r="AI122" s="118"/>
+      <c r="AJ122" s="118"/>
+      <c r="AK122" s="118"/>
+      <c r="AL122" s="118"/>
+      <c r="AM122" s="118"/>
+      <c r="AN122" s="119"/>
+    </row>
+    <row r="123" spans="1:40" ht="168">
+      <c r="A123" s="112" t="s">
+        <v>287</v>
+      </c>
+      <c r="B123" s="130" t="s">
+        <v>401</v>
+      </c>
+      <c r="C123" s="84" t="s">
+        <v>402</v>
+      </c>
+      <c r="D123" s="90" t="s">
+        <v>403</v>
+      </c>
+      <c r="E123" s="95"/>
+      <c r="F123" s="101" t="s">
+        <v>46</v>
+      </c>
+      <c r="G123" s="102">
+        <v>100</v>
+      </c>
+      <c r="H123" s="33">
+        <f>IF(OR(J123="",K123="",K123&lt;J123),0,NETWORKDAYS(J123,K123,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I123" s="76">
+        <v>46150</v>
+      </c>
+      <c r="J123" s="76">
+        <v>46150</v>
+      </c>
+      <c r="K123" s="76"/>
+      <c r="L123" s="76">
+        <v>46171</v>
+      </c>
+      <c r="M123" s="36">
+        <f ca="1">IF(OR(J123="",AND(L123="",TODAY()&lt;J123),AND(L123&lt;&gt;"",L123&lt;J123)),0,
+   IF(L123="",
+      NETWORKDAYS(J123,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J123,L123,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>15</v>
+      </c>
+      <c r="N123" s="76"/>
+      <c r="O123" s="41"/>
+      <c r="P123" s="41"/>
+      <c r="Q123" s="92" t="s">
+        <v>404</v>
+      </c>
+      <c r="R123" s="133" t="s">
+        <v>39</v>
+      </c>
+      <c r="S123" s="113"/>
+      <c r="T123" s="114"/>
+      <c r="U123" s="114"/>
+      <c r="V123" s="114"/>
+      <c r="W123" s="114"/>
+      <c r="X123" s="114"/>
+      <c r="Y123" s="114"/>
+      <c r="Z123" s="114"/>
+      <c r="AA123" s="114"/>
+      <c r="AB123" s="114"/>
+      <c r="AC123" s="114"/>
+      <c r="AD123" s="114"/>
+      <c r="AE123" s="114"/>
+      <c r="AF123" s="114"/>
+      <c r="AG123" s="114"/>
+      <c r="AH123" s="114"/>
+      <c r="AI123" s="114"/>
+      <c r="AJ123" s="114"/>
+      <c r="AK123" s="114"/>
+      <c r="AL123" s="114"/>
+      <c r="AM123" s="114"/>
+      <c r="AN123" s="115"/>
+    </row>
+    <row r="124" spans="1:40" ht="36">
+      <c r="A124" s="116" t="s">
+        <v>405</v>
+      </c>
+      <c r="B124" s="134" t="s">
+        <v>406</v>
+      </c>
+      <c r="C124" s="87" t="s">
+        <v>407</v>
+      </c>
+      <c r="D124" s="91" t="s">
+        <v>408</v>
+      </c>
+      <c r="E124" s="93"/>
+      <c r="F124" s="103" t="s">
+        <v>46</v>
+      </c>
+      <c r="G124" s="104">
+        <v>100</v>
+      </c>
+      <c r="H124" s="20">
+        <f>IF(OR(J124="",K124="",K124&lt;J124),0,NETWORKDAYS(J124,K124,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I124" s="68">
+        <v>46153</v>
+      </c>
+      <c r="J124" s="68">
+        <v>46153</v>
+      </c>
+      <c r="K124" s="44"/>
+      <c r="L124" s="68">
+        <v>46153</v>
+      </c>
+      <c r="M124" s="23">
+        <f ca="1">IF(OR(J124="",AND(L124="",TODAY()&lt;J124),AND(L124&lt;&gt;"",L124&lt;J124)),0,
+   IF(L124="",
+      NETWORKDAYS(J124,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J124,L124,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N124" s="44"/>
+      <c r="O124" s="44"/>
+      <c r="P124" s="44"/>
+      <c r="Q124" s="55" t="s">
+        <v>409</v>
+      </c>
+      <c r="R124" s="129" t="s">
+        <v>39</v>
+      </c>
+      <c r="S124" s="117"/>
+      <c r="T124" s="118"/>
+      <c r="U124" s="118"/>
+      <c r="V124" s="118"/>
+      <c r="W124" s="118"/>
+      <c r="X124" s="118"/>
+      <c r="Y124" s="118"/>
+      <c r="Z124" s="118"/>
+      <c r="AA124" s="118"/>
+      <c r="AB124" s="118"/>
+      <c r="AC124" s="118"/>
+      <c r="AD124" s="118"/>
+      <c r="AE124" s="118"/>
+      <c r="AF124" s="118"/>
+      <c r="AG124" s="118"/>
+      <c r="AH124" s="118"/>
+      <c r="AI124" s="118"/>
+      <c r="AJ124" s="118"/>
+      <c r="AK124" s="118"/>
+      <c r="AL124" s="118"/>
+      <c r="AM124" s="118"/>
+      <c r="AN124" s="119"/>
+    </row>
+    <row r="125" spans="1:40">
+      <c r="A125" s="112" t="s">
+        <v>287</v>
+      </c>
+      <c r="B125" s="130" t="s">
+        <v>410</v>
+      </c>
+      <c r="C125" s="84" t="s">
+        <v>204</v>
+      </c>
+      <c r="D125" s="90" t="s">
+        <v>390</v>
+      </c>
+      <c r="E125" s="95"/>
+      <c r="F125" s="101" t="s">
+        <v>46</v>
+      </c>
+      <c r="G125" s="102">
+        <v>100</v>
+      </c>
+      <c r="H125" s="33">
+        <f>IF(OR(J125="",K125="",K125&lt;J125),0,NETWORKDAYS(J125,K125,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I125" s="76">
+        <v>46154</v>
+      </c>
+      <c r="J125" s="76"/>
+      <c r="K125" s="76"/>
+      <c r="L125" s="76">
+        <v>46154</v>
+      </c>
+      <c r="M125" s="36">
+        <f ca="1">IF(OR(J125="",AND(L125="",TODAY()&lt;J125),AND(L125&lt;&gt;"",L125&lt;J125)),0,
+   IF(L125="",
+      NETWORKDAYS(J125,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J125,L125,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
+      </c>
+      <c r="N125" s="41"/>
+      <c r="O125" s="41"/>
+      <c r="P125" s="41"/>
+      <c r="Q125" s="92" t="s">
+        <v>411</v>
+      </c>
+      <c r="R125" s="133" t="s">
+        <v>39</v>
+      </c>
+      <c r="S125" s="113"/>
+      <c r="T125" s="114"/>
+      <c r="U125" s="114"/>
+      <c r="V125" s="114"/>
+      <c r="W125" s="114"/>
+      <c r="X125" s="114"/>
+      <c r="Y125" s="114"/>
+      <c r="Z125" s="114"/>
+      <c r="AA125" s="114"/>
+      <c r="AB125" s="114"/>
+      <c r="AC125" s="114"/>
+      <c r="AD125" s="114"/>
+      <c r="AE125" s="114"/>
+      <c r="AF125" s="114"/>
+      <c r="AG125" s="114"/>
+      <c r="AH125" s="114"/>
+      <c r="AI125" s="114"/>
+      <c r="AJ125" s="114"/>
+      <c r="AK125" s="114"/>
+      <c r="AL125" s="114"/>
+      <c r="AM125" s="114"/>
+      <c r="AN125" s="115"/>
+    </row>
+    <row r="126" spans="1:40" ht="25.5">
+      <c r="A126" s="116" t="s">
+        <v>287</v>
+      </c>
+      <c r="B126" s="134" t="s">
+        <v>412</v>
+      </c>
+      <c r="C126" s="87" t="s">
+        <v>413</v>
+      </c>
+      <c r="D126" s="91" t="s">
+        <v>414</v>
+      </c>
+      <c r="E126" s="93"/>
+      <c r="F126" s="103" t="s">
+        <v>46</v>
+      </c>
+      <c r="G126" s="104">
+        <v>0</v>
+      </c>
+      <c r="H126" s="20">
+        <f>IF(OR(J126="",K126="",K126&lt;J126),0,NETWORKDAYS(J126,K126,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I126" s="68">
+        <v>46154</v>
+      </c>
+      <c r="J126" s="68"/>
+      <c r="K126" s="68"/>
+      <c r="L126" s="68">
+        <v>46154</v>
+      </c>
+      <c r="M126" s="23">
+        <f ca="1">IF(OR(J126="",AND(L126="",TODAY()&lt;J126),AND(L126&lt;&gt;"",L126&lt;J126)),0,
+   IF(L126="",
+      NETWORKDAYS(J126,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J126,L126,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
+      </c>
+      <c r="N126" s="44"/>
+      <c r="O126" s="44"/>
+      <c r="P126" s="44"/>
+      <c r="Q126" s="55" t="s">
+        <v>415</v>
+      </c>
+      <c r="R126" s="129" t="s">
+        <v>39</v>
+      </c>
+      <c r="S126" s="117"/>
+      <c r="T126" s="118"/>
+      <c r="U126" s="118"/>
+      <c r="V126" s="118"/>
+      <c r="W126" s="118"/>
+      <c r="X126" s="118"/>
+      <c r="Y126" s="118"/>
+      <c r="Z126" s="118"/>
+      <c r="AA126" s="118"/>
+      <c r="AB126" s="118"/>
+      <c r="AC126" s="118"/>
+      <c r="AD126" s="118"/>
+      <c r="AE126" s="118"/>
+      <c r="AF126" s="118"/>
+      <c r="AG126" s="118"/>
+      <c r="AH126" s="118"/>
+      <c r="AI126" s="118"/>
+      <c r="AJ126" s="118"/>
+      <c r="AK126" s="118"/>
+      <c r="AL126" s="118"/>
+      <c r="AM126" s="118"/>
+      <c r="AN126" s="119"/>
+    </row>
+    <row r="127" spans="1:40">
+      <c r="A127" s="112" t="s">
+        <v>18</v>
+      </c>
+      <c r="B127" s="130" t="s">
+        <v>416</v>
+      </c>
+      <c r="C127" s="84" t="s">
+        <v>417</v>
+      </c>
+      <c r="D127" s="90" t="s">
+        <v>418</v>
+      </c>
+      <c r="E127" s="95"/>
+      <c r="F127" s="101" t="s">
+        <v>46</v>
+      </c>
+      <c r="G127" s="102">
+        <v>100</v>
+      </c>
+      <c r="H127" s="33">
+        <f>IF(OR(J127="",K127="",K127&lt;J127),0,NETWORKDAYS(J127,K127,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I127" s="76">
+        <v>46155</v>
+      </c>
+      <c r="J127" s="41"/>
+      <c r="K127" s="41"/>
+      <c r="L127" s="76">
+        <v>46156</v>
+      </c>
+      <c r="M127" s="36">
+        <f ca="1">IF(OR(J127="",AND(L127="",TODAY()&lt;J127),AND(L127&lt;&gt;"",L127&lt;J127)),0,
+   IF(L127="",
+      NETWORKDAYS(J127,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J127,L127,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
+      </c>
+      <c r="N127" s="41"/>
+      <c r="O127" s="41"/>
+      <c r="P127" s="41"/>
+      <c r="Q127" s="92" t="s">
+        <v>419</v>
+      </c>
+      <c r="R127" s="133" t="s">
+        <v>39</v>
+      </c>
+      <c r="S127" s="106"/>
+      <c r="T127" s="107"/>
+      <c r="U127" s="107"/>
+      <c r="V127" s="107"/>
+      <c r="W127" s="107"/>
+      <c r="X127" s="107"/>
+      <c r="Y127" s="107"/>
+      <c r="Z127" s="107"/>
+      <c r="AA127" s="107"/>
+      <c r="AB127" s="107"/>
+      <c r="AC127" s="107"/>
+      <c r="AD127" s="107"/>
+      <c r="AE127" s="107"/>
+      <c r="AF127" s="107"/>
+      <c r="AG127" s="107"/>
+      <c r="AH127" s="107"/>
+      <c r="AI127" s="107"/>
+      <c r="AJ127" s="107"/>
+      <c r="AK127" s="107"/>
+      <c r="AL127" s="107"/>
+      <c r="AM127" s="107"/>
+      <c r="AN127" s="108"/>
+    </row>
+    <row r="128" spans="1:40" ht="60">
+      <c r="A128" s="116" t="s">
+        <v>287</v>
+      </c>
+      <c r="B128" s="134" t="s">
+        <v>420</v>
+      </c>
+      <c r="C128" s="87" t="s">
+        <v>421</v>
+      </c>
+      <c r="D128" s="91" t="s">
+        <v>422</v>
+      </c>
+      <c r="E128" s="93"/>
+      <c r="F128" s="103" t="s">
+        <v>46</v>
+      </c>
+      <c r="G128" s="104">
+        <v>100</v>
+      </c>
+      <c r="H128" s="20">
+        <f>IF(OR(J128="",K128="",K128&lt;J128),0,NETWORKDAYS(J128,K128,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I128" s="68">
+        <v>46156</v>
+      </c>
+      <c r="J128" s="68">
+        <v>46162</v>
+      </c>
+      <c r="K128" s="44"/>
+      <c r="L128" s="68">
+        <v>46162</v>
+      </c>
+      <c r="M128" s="23">
+        <f ca="1">IF(OR(J128="",AND(L128="",TODAY()&lt;J128),AND(L128&lt;&gt;"",L128&lt;J128)),0,
+   IF(L128="",
+      NETWORKDAYS(J128,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J128,L128,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N128" s="44"/>
+      <c r="O128" s="44"/>
+      <c r="P128" s="44"/>
+      <c r="Q128" s="55" t="s">
+        <v>423</v>
+      </c>
+      <c r="R128" s="129" t="s">
+        <v>39</v>
+      </c>
+      <c r="S128" s="117"/>
+      <c r="T128" s="118"/>
+      <c r="U128" s="118"/>
+      <c r="V128" s="118"/>
+      <c r="W128" s="118"/>
+      <c r="X128" s="118"/>
+      <c r="Y128" s="118"/>
+      <c r="Z128" s="118"/>
+      <c r="AA128" s="118"/>
+      <c r="AB128" s="118"/>
+      <c r="AC128" s="118"/>
+      <c r="AD128" s="118"/>
+      <c r="AE128" s="118"/>
+      <c r="AF128" s="118"/>
+      <c r="AG128" s="118"/>
+      <c r="AH128" s="118"/>
+      <c r="AI128" s="118"/>
+      <c r="AJ128" s="118"/>
+      <c r="AK128" s="118"/>
+      <c r="AL128" s="118"/>
+      <c r="AM128" s="118"/>
+      <c r="AN128" s="119"/>
+    </row>
+    <row r="129" spans="1:40" ht="36">
+      <c r="A129" s="112" t="s">
+        <v>18</v>
+      </c>
+      <c r="B129" s="130" t="s">
+        <v>424</v>
+      </c>
+      <c r="C129" s="84" t="s">
+        <v>315</v>
+      </c>
+      <c r="D129" s="90" t="s">
+        <v>316</v>
+      </c>
+      <c r="E129" s="95"/>
+      <c r="F129" s="101" t="s">
+        <v>46</v>
+      </c>
+      <c r="G129" s="102">
+        <v>100</v>
+      </c>
+      <c r="H129" s="33">
+        <f>IF(OR(J129="",K129="",K129&lt;J129),0,NETWORKDAYS(J129,K129,Hoja2!$A$2:$A$53))</f>
+        <v>2</v>
+      </c>
+      <c r="I129" s="76">
+        <v>46162</v>
+      </c>
+      <c r="J129" s="76">
+        <v>46169</v>
+      </c>
+      <c r="K129" s="76">
+        <v>46170</v>
+      </c>
+      <c r="L129" s="76">
+        <v>46169</v>
+      </c>
+      <c r="M129" s="36">
+        <f ca="1">IF(OR(J129="",AND(L129="",TODAY()&lt;J129),AND(L129&lt;&gt;"",L129&lt;J129)),0,
+   IF(L129="",
+      NETWORKDAYS(J129,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J129,L129,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N129" s="76">
+        <v>46170</v>
+      </c>
+      <c r="O129" s="41"/>
+      <c r="P129" s="41"/>
+      <c r="Q129" s="92" t="s">
+        <v>425</v>
+      </c>
+      <c r="R129" s="133" t="s">
+        <v>39</v>
+      </c>
+      <c r="S129" s="113"/>
+      <c r="T129" s="114"/>
+      <c r="U129" s="114"/>
+      <c r="V129" s="114"/>
+      <c r="W129" s="114"/>
+      <c r="X129" s="114"/>
+      <c r="Y129" s="114"/>
+      <c r="Z129" s="114"/>
+      <c r="AA129" s="114"/>
+      <c r="AB129" s="114"/>
+      <c r="AC129" s="114"/>
+      <c r="AD129" s="114"/>
+      <c r="AE129" s="114"/>
+      <c r="AF129" s="114"/>
+      <c r="AG129" s="114"/>
+      <c r="AH129" s="114"/>
+      <c r="AI129" s="114"/>
+      <c r="AJ129" s="114"/>
+      <c r="AK129" s="114"/>
+      <c r="AL129" s="114"/>
+      <c r="AM129" s="114"/>
+      <c r="AN129" s="115"/>
+    </row>
+    <row r="130" spans="1:40">
+      <c r="A130" s="116" t="s">
+        <v>18</v>
+      </c>
+      <c r="B130" s="134" t="s">
+        <v>426</v>
+      </c>
+      <c r="C130" s="87" t="s">
+        <v>204</v>
+      </c>
+      <c r="D130" s="91" t="s">
+        <v>390</v>
+      </c>
+      <c r="E130" s="93"/>
+      <c r="F130" s="103" t="s">
+        <v>46</v>
+      </c>
+      <c r="G130" s="104">
+        <v>100</v>
+      </c>
+      <c r="H130" s="20">
+        <f>IF(OR(J130="",K130="",K130&lt;J130),0,NETWORKDAYS(J130,K130,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I130" s="68">
+        <v>46167</v>
+      </c>
+      <c r="J130" s="68">
+        <v>46167</v>
+      </c>
+      <c r="K130" s="44"/>
+      <c r="L130" s="68">
+        <v>46167</v>
+      </c>
+      <c r="M130" s="23">
+        <f ca="1">IF(OR(J130="",AND(L130="",TODAY()&lt;J130),AND(L130&lt;&gt;"",L130&lt;J130)),0,
+   IF(L130="",
+      NETWORKDAYS(J130,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J130,L130,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N130" s="44"/>
+      <c r="O130" s="44"/>
+      <c r="P130" s="44"/>
+      <c r="Q130" s="55" t="s">
+        <v>427</v>
+      </c>
+      <c r="R130" s="129" t="s">
+        <v>39</v>
+      </c>
+      <c r="S130" s="117"/>
+      <c r="T130" s="118"/>
+      <c r="U130" s="118"/>
+      <c r="V130" s="118"/>
+      <c r="W130" s="118"/>
+      <c r="X130" s="118"/>
+      <c r="Y130" s="118"/>
+      <c r="Z130" s="118"/>
+      <c r="AA130" s="118"/>
+      <c r="AB130" s="118"/>
+      <c r="AC130" s="118"/>
+      <c r="AD130" s="118"/>
+      <c r="AE130" s="118"/>
+      <c r="AF130" s="118"/>
+      <c r="AG130" s="118"/>
+      <c r="AH130" s="118"/>
+      <c r="AI130" s="118"/>
+      <c r="AJ130" s="118"/>
+      <c r="AK130" s="118"/>
+      <c r="AL130" s="118"/>
+      <c r="AM130" s="118"/>
+      <c r="AN130" s="119"/>
+    </row>
+    <row r="131" spans="1:40" ht="36">
+      <c r="A131" s="112" t="s">
+        <v>287</v>
+      </c>
+      <c r="B131" s="130" t="s">
+        <v>428</v>
+      </c>
+      <c r="C131" s="84" t="s">
+        <v>413</v>
+      </c>
+      <c r="D131" s="90" t="s">
+        <v>429</v>
+      </c>
+      <c r="E131" s="95"/>
+      <c r="F131" s="101" t="s">
+        <v>46</v>
+      </c>
+      <c r="G131" s="102">
+        <v>100</v>
+      </c>
+      <c r="H131" s="33">
+        <f>IF(OR(J131="",K131="",K131&lt;J131),0,NETWORKDAYS(J131,K131,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I131" s="137">
+        <v>46168</v>
+      </c>
+      <c r="J131" s="76">
+        <v>46171</v>
+      </c>
+      <c r="K131" s="76"/>
+      <c r="L131" s="76">
+        <v>46171</v>
+      </c>
+      <c r="M131" s="36">
+        <f ca="1">IF(OR(J131="",AND(L131="",TODAY()&lt;J131),AND(L131&lt;&gt;"",L131&lt;J131)),0,
+   IF(L131="",
+      NETWORKDAYS(J131,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J131,L131,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N131" s="41"/>
+      <c r="O131" s="41"/>
+      <c r="P131" s="41"/>
+      <c r="Q131" s="92" t="s">
+        <v>430</v>
+      </c>
+      <c r="R131" s="133" t="s">
+        <v>39</v>
+      </c>
+      <c r="S131" s="113"/>
+      <c r="T131" s="114"/>
+      <c r="U131" s="114"/>
+      <c r="V131" s="114"/>
+      <c r="W131" s="114"/>
+      <c r="X131" s="114"/>
+      <c r="Y131" s="114"/>
+      <c r="Z131" s="114"/>
+      <c r="AA131" s="114"/>
+      <c r="AB131" s="114"/>
+      <c r="AC131" s="114"/>
+      <c r="AD131" s="114"/>
+      <c r="AE131" s="114"/>
+      <c r="AF131" s="114"/>
+      <c r="AG131" s="114"/>
+      <c r="AH131" s="114"/>
+      <c r="AI131" s="114"/>
+      <c r="AJ131" s="114"/>
+      <c r="AK131" s="114"/>
+      <c r="AL131" s="114"/>
+      <c r="AM131" s="114"/>
+      <c r="AN131" s="115"/>
+    </row>
+    <row r="132" spans="1:40">
+      <c r="A132" s="116" t="s">
+        <v>287</v>
+      </c>
+      <c r="B132" s="134" t="s">
+        <v>431</v>
+      </c>
+      <c r="C132" s="87" t="s">
+        <v>204</v>
+      </c>
+      <c r="D132" s="91" t="s">
+        <v>390</v>
+      </c>
+      <c r="E132" s="93"/>
+      <c r="F132" s="103" t="s">
+        <v>46</v>
+      </c>
+      <c r="G132" s="104">
+        <v>100</v>
+      </c>
+      <c r="H132" s="20">
+        <f>IF(OR(J132="",K132="",K132&lt;J132),0,NETWORKDAYS(J132,K132,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I132" s="68">
+        <v>46169</v>
+      </c>
+      <c r="J132" s="68">
+        <v>46169</v>
+      </c>
+      <c r="K132" s="44"/>
+      <c r="L132" s="68">
+        <v>46169</v>
+      </c>
+      <c r="M132" s="23">
+        <f ca="1">IF(OR(J132="",AND(L132="",TODAY()&lt;J132),AND(L132&lt;&gt;"",L132&lt;J132)),0,
+   IF(L132="",
+      NETWORKDAYS(J132,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J132,L132,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N132" s="44"/>
+      <c r="O132" s="44"/>
+      <c r="P132" s="44"/>
+      <c r="Q132" s="55" t="s">
+        <v>432</v>
+      </c>
+      <c r="R132" s="129" t="s">
+        <v>39</v>
+      </c>
+      <c r="S132" s="109"/>
+      <c r="T132" s="110"/>
+      <c r="U132" s="110"/>
+      <c r="V132" s="110"/>
+      <c r="W132" s="110"/>
+      <c r="X132" s="110"/>
+      <c r="Y132" s="110"/>
+      <c r="Z132" s="110"/>
+      <c r="AA132" s="110"/>
+      <c r="AB132" s="110"/>
+      <c r="AC132" s="110"/>
+      <c r="AD132" s="110"/>
+      <c r="AE132" s="110"/>
+      <c r="AF132" s="110"/>
+      <c r="AG132" s="110"/>
+      <c r="AH132" s="110"/>
+      <c r="AI132" s="110"/>
+      <c r="AJ132" s="110"/>
+      <c r="AK132" s="110"/>
+      <c r="AL132" s="110"/>
+      <c r="AM132" s="110"/>
+      <c r="AN132" s="111"/>
+    </row>
+    <row r="133" spans="1:40">
+      <c r="A133" s="112" t="s">
+        <v>287</v>
+      </c>
+      <c r="B133" s="130" t="s">
+        <v>433</v>
+      </c>
+      <c r="C133" s="84" t="s">
+        <v>434</v>
+      </c>
+      <c r="D133" s="90" t="s">
+        <v>435</v>
+      </c>
+      <c r="E133" s="95"/>
+      <c r="F133" s="101" t="s">
+        <v>46</v>
+      </c>
+      <c r="G133" s="102">
+        <v>100</v>
+      </c>
+      <c r="H133" s="33">
+        <f>IF(OR(J133="",K133="",K133&lt;J133),0,NETWORKDAYS(J133,K133,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I133" s="76">
+        <v>46174</v>
+      </c>
+      <c r="J133" s="76">
+        <v>46174</v>
+      </c>
+      <c r="K133" s="41"/>
+      <c r="L133" s="76">
+        <v>46174</v>
+      </c>
+      <c r="M133" s="36">
+        <f ca="1">IF(OR(J133="",AND(L133="",TODAY()&lt;J133),AND(L133&lt;&gt;"",L133&lt;J133)),0,
+   IF(L133="",
+      NETWORKDAYS(J133,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J133,L133,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N133" s="41"/>
+      <c r="O133" s="41"/>
+      <c r="P133" s="41"/>
+      <c r="Q133" s="92" t="s">
+        <v>436</v>
+      </c>
+      <c r="R133" s="133" t="s">
+        <v>39</v>
+      </c>
+      <c r="S133" s="106"/>
+      <c r="T133" s="107"/>
+      <c r="U133" s="107"/>
+      <c r="V133" s="107"/>
+      <c r="W133" s="107"/>
+      <c r="X133" s="107"/>
+      <c r="Y133" s="107"/>
+      <c r="Z133" s="107"/>
+      <c r="AA133" s="107"/>
+      <c r="AB133" s="107"/>
+      <c r="AC133" s="107"/>
+      <c r="AD133" s="107"/>
+      <c r="AE133" s="107"/>
+      <c r="AF133" s="107"/>
+      <c r="AG133" s="107"/>
+      <c r="AH133" s="107"/>
+      <c r="AI133" s="107"/>
+      <c r="AJ133" s="107"/>
+      <c r="AK133" s="107"/>
+      <c r="AL133" s="107"/>
+      <c r="AM133" s="107"/>
+      <c r="AN133" s="108"/>
+    </row>
+    <row r="134" spans="1:40" ht="24">
+      <c r="A134" s="116" t="s">
+        <v>287</v>
+      </c>
+      <c r="B134" s="134" t="s">
+        <v>437</v>
+      </c>
+      <c r="C134" s="87" t="s">
+        <v>204</v>
+      </c>
+      <c r="D134" s="91" t="s">
+        <v>390</v>
+      </c>
+      <c r="E134" s="93"/>
+      <c r="F134" s="103" t="s">
+        <v>46</v>
+      </c>
+      <c r="G134" s="104">
+        <v>100</v>
+      </c>
+      <c r="H134" s="20">
+        <f>IF(OR(J134="",K134="",K134&lt;J134),0,NETWORKDAYS(J134,K134,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I134" s="68">
+        <v>46175</v>
+      </c>
+      <c r="J134" s="68">
+        <v>46175</v>
+      </c>
+      <c r="K134" s="44"/>
+      <c r="L134" s="68">
+        <v>46175</v>
+      </c>
+      <c r="M134" s="23">
+        <f ca="1">IF(OR(J134="",AND(L134="",TODAY()&lt;J134),AND(L134&lt;&gt;"",L134&lt;J134)),0,
+   IF(L134="",
+      NETWORKDAYS(J134,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J134,L134,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N134" s="44"/>
+      <c r="O134" s="44"/>
+      <c r="P134" s="44"/>
+      <c r="Q134" s="55" t="s">
+        <v>438</v>
+      </c>
+      <c r="R134" s="129" t="s">
+        <v>39</v>
+      </c>
+      <c r="S134" s="109"/>
+      <c r="T134" s="110"/>
+      <c r="U134" s="110"/>
+      <c r="V134" s="110"/>
+      <c r="W134" s="110"/>
+      <c r="X134" s="110"/>
+      <c r="Y134" s="110"/>
+      <c r="Z134" s="110"/>
+      <c r="AA134" s="110"/>
+      <c r="AB134" s="110"/>
+      <c r="AC134" s="110"/>
+      <c r="AD134" s="110"/>
+      <c r="AE134" s="110"/>
+      <c r="AF134" s="110"/>
+      <c r="AG134" s="110"/>
+      <c r="AH134" s="110"/>
+      <c r="AI134" s="110"/>
+      <c r="AJ134" s="110"/>
+      <c r="AK134" s="110"/>
+      <c r="AL134" s="110"/>
+      <c r="AM134" s="110"/>
+      <c r="AN134" s="111"/>
+    </row>
+    <row r="135" spans="1:40">
+      <c r="A135" s="112" t="s">
+        <v>18</v>
+      </c>
+      <c r="B135" s="130" t="s">
+        <v>439</v>
+      </c>
+      <c r="C135" s="131" t="s">
+        <v>440</v>
+      </c>
+      <c r="D135" s="90" t="s">
+        <v>441</v>
+      </c>
+      <c r="E135" s="95"/>
+      <c r="F135" s="101" t="s">
+        <v>46</v>
+      </c>
+      <c r="G135" s="102">
+        <v>100</v>
+      </c>
+      <c r="H135" s="33">
+        <f>IF(OR(J135="",K135="",K135&lt;J135),0,NETWORKDAYS(J135,K135,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I135" s="76">
+        <v>46177</v>
+      </c>
+      <c r="J135" s="76">
+        <v>46177</v>
+      </c>
+      <c r="K135" s="41"/>
+      <c r="L135" s="76">
+        <v>46177</v>
+      </c>
+      <c r="M135" s="36">
+        <f ca="1">IF(OR(J135="",AND(L135="",TODAY()&lt;J135),AND(L135&lt;&gt;"",L135&lt;J135)),0,
+   IF(L135="",
+      NETWORKDAYS(J135,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J135,L135,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N135" s="41"/>
+      <c r="O135" s="41"/>
+      <c r="P135" s="41"/>
+      <c r="Q135" s="92" t="s">
+        <v>442</v>
+      </c>
+      <c r="R135" s="133" t="s">
+        <v>39</v>
+      </c>
+      <c r="S135" s="113"/>
+      <c r="T135" s="114"/>
+      <c r="U135" s="114"/>
+      <c r="V135" s="114"/>
+      <c r="W135" s="114"/>
+      <c r="X135" s="114"/>
+      <c r="Y135" s="114"/>
+      <c r="Z135" s="114"/>
+      <c r="AA135" s="114"/>
+      <c r="AB135" s="114"/>
+      <c r="AC135" s="114"/>
+      <c r="AD135" s="114"/>
+      <c r="AE135" s="114"/>
+      <c r="AF135" s="114"/>
+      <c r="AG135" s="114"/>
+      <c r="AH135" s="114"/>
+      <c r="AI135" s="114"/>
+      <c r="AJ135" s="114"/>
+      <c r="AK135" s="114"/>
+      <c r="AL135" s="114"/>
+      <c r="AM135" s="114"/>
+      <c r="AN135" s="115"/>
+    </row>
+    <row r="136" spans="1:40" ht="25.5">
+      <c r="A136" s="116" t="s">
+        <v>18</v>
+      </c>
+      <c r="B136" s="134" t="s">
+        <v>443</v>
+      </c>
+      <c r="C136" s="127" t="s">
+        <v>444</v>
+      </c>
+      <c r="D136" s="91" t="s">
+        <v>445</v>
+      </c>
+      <c r="E136" s="93"/>
+      <c r="F136" s="103" t="s">
+        <v>251</v>
+      </c>
+      <c r="G136" s="104">
+        <v>0</v>
+      </c>
+      <c r="H136" s="20">
+        <f>IF(OR(J136="",K136="",K136&lt;J136),0,NETWORKDAYS(J136,K136,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I136" s="68">
+        <v>46177</v>
+      </c>
+      <c r="J136" s="44"/>
+      <c r="K136" s="44"/>
+      <c r="L136" s="44"/>
+      <c r="M136" s="23">
+        <f ca="1">IF(OR(J136="",AND(L136="",TODAY()&lt;J136),AND(L136&lt;&gt;"",L136&lt;J136)),0,
+   IF(L136="",
+      NETWORKDAYS(J136,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J136,L136,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
+      </c>
+      <c r="N136" s="68">
+        <v>46183</v>
+      </c>
+      <c r="O136" s="44"/>
+      <c r="P136" s="44"/>
+      <c r="Q136" s="55" t="s">
+        <v>446</v>
+      </c>
+      <c r="R136" s="133" t="s">
+        <v>39</v>
+      </c>
+      <c r="S136" s="109"/>
+      <c r="T136" s="110"/>
+      <c r="U136" s="110"/>
+      <c r="V136" s="110"/>
+      <c r="W136" s="110"/>
+      <c r="X136" s="110"/>
+      <c r="Y136" s="110"/>
+      <c r="Z136" s="110"/>
+      <c r="AA136" s="110"/>
+      <c r="AB136" s="110"/>
+      <c r="AC136" s="110"/>
+      <c r="AD136" s="110"/>
+      <c r="AE136" s="110"/>
+      <c r="AF136" s="110"/>
+      <c r="AG136" s="110"/>
+      <c r="AH136" s="110"/>
+      <c r="AI136" s="110"/>
+      <c r="AJ136" s="110"/>
+      <c r="AK136" s="110"/>
+      <c r="AL136" s="110"/>
+      <c r="AM136" s="110"/>
+      <c r="AN136" s="111"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AN106"/>
-  <conditionalFormatting sqref="B2:B106">
+  <autoFilter ref="A1:AN136"/>
+  <conditionalFormatting sqref="B2:B136">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>COUNTIF(B$2:B$16,B2)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="I2:L9 J10:L10 I11:L54 N2:P54 I56:L106 N56:P106">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="I2:L9 J10:L10 I11:L54 N2:P54 I56:L136 N56:P136">
       <formula1>OR(NOT(ISERROR(DATEVALUE(I2))), AND(ISNUMBER(I2), LEFT(CELL("format", I2))="D"))</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F106">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F136">
       <formula1>"FINALIZADO,EN PROCESO,PAUSADO,EN TEST,PENDIENTE,PRUEBAS CLIENTE,PRUEBAS IMAGINE,PASO A PRODUCCION"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10244,427 +12846,427 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A1" s="136">
+      <c r="A1" s="138">
         <v>45292</v>
       </c>
-      <c r="B1" s="137" t="s">
-        <v>346</v>
+      <c r="B1" s="139" t="s">
+        <v>447</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A2" s="136">
+      <c r="A2" s="138">
         <v>45299</v>
       </c>
-      <c r="B2" s="137" t="s">
-        <v>347</v>
+      <c r="B2" s="139" t="s">
+        <v>448</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A3" s="136">
+      <c r="A3" s="138">
         <v>45376</v>
       </c>
-      <c r="B3" s="137" t="s">
-        <v>348</v>
+      <c r="B3" s="139" t="s">
+        <v>449</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A4" s="136">
+      <c r="A4" s="138">
         <v>45379</v>
       </c>
-      <c r="B4" s="137" t="s">
-        <v>349</v>
+      <c r="B4" s="139" t="s">
+        <v>450</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A5" s="136">
+      <c r="A5" s="138">
         <v>45380</v>
       </c>
-      <c r="B5" s="137" t="s">
-        <v>350</v>
+      <c r="B5" s="139" t="s">
+        <v>451</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A6" s="136">
+      <c r="A6" s="138">
         <v>45413</v>
       </c>
-      <c r="B6" s="137" t="s">
-        <v>351</v>
+      <c r="B6" s="139" t="s">
+        <v>452</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A7" s="136">
+      <c r="A7" s="138">
         <v>45425</v>
       </c>
-      <c r="B7" s="137" t="s">
-        <v>352</v>
+      <c r="B7" s="139" t="s">
+        <v>453</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A8" s="136">
+      <c r="A8" s="138">
         <v>45446</v>
       </c>
-      <c r="B8" s="137" t="s">
-        <v>353</v>
+      <c r="B8" s="139" t="s">
+        <v>454</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A9" s="136">
+      <c r="A9" s="138">
         <v>45453</v>
       </c>
-      <c r="B9" s="137" t="s">
-        <v>354</v>
+      <c r="B9" s="139" t="s">
+        <v>455</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A10" s="136">
+      <c r="A10" s="138">
         <v>45474</v>
       </c>
-      <c r="B10" s="137" t="s">
-        <v>355</v>
+      <c r="B10" s="139" t="s">
+        <v>456</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A11" s="136">
+      <c r="A11" s="138">
         <v>45493</v>
       </c>
-      <c r="B11" s="137" t="s">
-        <v>356</v>
+      <c r="B11" s="139" t="s">
+        <v>457</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A12" s="136">
+      <c r="A12" s="138">
         <v>45511</v>
       </c>
-      <c r="B12" s="137" t="s">
-        <v>357</v>
+      <c r="B12" s="139" t="s">
+        <v>458</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A13" s="136">
+      <c r="A13" s="138">
         <v>45523</v>
       </c>
-      <c r="B13" s="137" t="s">
-        <v>358</v>
+      <c r="B13" s="139" t="s">
+        <v>459</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A14" s="136">
+      <c r="A14" s="138">
         <v>45579</v>
       </c>
-      <c r="B14" s="137" t="s">
-        <v>359</v>
+      <c r="B14" s="139" t="s">
+        <v>460</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A15" s="136">
+      <c r="A15" s="138">
         <v>45600</v>
       </c>
-      <c r="B15" s="137" t="s">
-        <v>360</v>
+      <c r="B15" s="139" t="s">
+        <v>461</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A16" s="136">
+      <c r="A16" s="138">
         <v>45607</v>
       </c>
-      <c r="B16" s="137" t="s">
-        <v>361</v>
+      <c r="B16" s="139" t="s">
+        <v>462</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A17" s="136">
+      <c r="A17" s="138">
         <v>45634</v>
       </c>
-      <c r="B17" s="137" t="s">
-        <v>362</v>
+      <c r="B17" s="139" t="s">
+        <v>463</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A18" s="136">
+      <c r="A18" s="138">
         <v>45651</v>
       </c>
-      <c r="B18" s="137" t="s">
-        <v>363</v>
+      <c r="B18" s="139" t="s">
+        <v>464</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A19" s="136">
+      <c r="A19" s="138">
         <v>45658</v>
       </c>
-      <c r="B19" s="138" t="s">
-        <v>364</v>
+      <c r="B19" s="140" t="s">
+        <v>465</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A20" s="136">
+      <c r="A20" s="138">
         <v>45663</v>
       </c>
-      <c r="B20" s="138" t="s">
-        <v>365</v>
+      <c r="B20" s="140" t="s">
+        <v>466</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A21" s="136">
+      <c r="A21" s="138">
         <v>45740</v>
       </c>
-      <c r="B21" s="138" t="s">
-        <v>366</v>
+      <c r="B21" s="140" t="s">
+        <v>467</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A22" s="136">
+      <c r="A22" s="138">
         <v>45764</v>
       </c>
-      <c r="B22" s="138" t="s">
-        <v>367</v>
+      <c r="B22" s="140" t="s">
+        <v>468</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A23" s="136">
+      <c r="A23" s="138">
         <v>45765</v>
       </c>
-      <c r="B23" s="138" t="s">
-        <v>368</v>
+      <c r="B23" s="140" t="s">
+        <v>469</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A24" s="136">
+      <c r="A24" s="138">
         <v>45778</v>
       </c>
-      <c r="B24" s="138" t="s">
-        <v>369</v>
+      <c r="B24" s="140" t="s">
+        <v>470</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A25" s="136">
+      <c r="A25" s="138">
         <v>45810</v>
       </c>
-      <c r="B25" s="138" t="s">
-        <v>370</v>
+      <c r="B25" s="140" t="s">
+        <v>471</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A26" s="136">
+      <c r="A26" s="138">
         <v>45831</v>
       </c>
-      <c r="B26" s="138" t="s">
-        <v>371</v>
+      <c r="B26" s="140" t="s">
+        <v>472</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A27" s="136">
+      <c r="A27" s="138">
         <v>45838</v>
       </c>
-      <c r="B27" s="138" t="s">
-        <v>372</v>
+      <c r="B27" s="140" t="s">
+        <v>473</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A28" s="136">
+      <c r="A28" s="138">
         <v>45858</v>
       </c>
-      <c r="B28" s="138" t="s">
-        <v>373</v>
+      <c r="B28" s="140" t="s">
+        <v>474</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A29" s="136">
+      <c r="A29" s="138">
         <v>45876</v>
       </c>
-      <c r="B29" s="138" t="s">
-        <v>374</v>
+      <c r="B29" s="140" t="s">
+        <v>475</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A30" s="136">
+      <c r="A30" s="138">
         <v>45887</v>
       </c>
-      <c r="B30" s="138" t="s">
-        <v>375</v>
+      <c r="B30" s="140" t="s">
+        <v>476</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A31" s="136">
+      <c r="A31" s="138">
         <v>45943</v>
       </c>
-      <c r="B31" s="138" t="s">
-        <v>376</v>
+      <c r="B31" s="140" t="s">
+        <v>477</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A32" s="136">
+      <c r="A32" s="138">
         <v>45964</v>
       </c>
-      <c r="B32" s="138" t="s">
-        <v>377</v>
+      <c r="B32" s="140" t="s">
+        <v>478</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A33" s="136">
+      <c r="A33" s="138">
         <v>45978</v>
       </c>
-      <c r="B33" s="138" t="s">
-        <v>378</v>
+      <c r="B33" s="140" t="s">
+        <v>479</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A34" s="136">
+      <c r="A34" s="138">
         <v>45999</v>
       </c>
-      <c r="B34" s="138" t="s">
-        <v>379</v>
+      <c r="B34" s="140" t="s">
+        <v>480</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A35" s="136">
+      <c r="A35" s="138">
         <v>46016</v>
       </c>
-      <c r="B35" s="138" t="s">
-        <v>380</v>
+      <c r="B35" s="140" t="s">
+        <v>481</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A36" s="136">
+      <c r="A36" s="138">
         <v>46023</v>
       </c>
-      <c r="B36" s="138" t="s">
-        <v>364</v>
+      <c r="B36" s="140" t="s">
+        <v>465</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A37" s="136">
+      <c r="A37" s="138">
         <v>46034</v>
       </c>
-      <c r="B37" s="138" t="s">
-        <v>365</v>
+      <c r="B37" s="140" t="s">
+        <v>466</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A38" s="136">
+      <c r="A38" s="138">
         <v>46104</v>
       </c>
-      <c r="B38" s="138" t="s">
-        <v>366</v>
+      <c r="B38" s="140" t="s">
+        <v>467</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A39" s="136">
+      <c r="A39" s="138">
         <v>46114</v>
       </c>
-      <c r="B39" s="138" t="s">
-        <v>367</v>
+      <c r="B39" s="140" t="s">
+        <v>468</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A40" s="136">
+      <c r="A40" s="138">
         <v>46115</v>
       </c>
-      <c r="B40" s="138" t="s">
-        <v>368</v>
+      <c r="B40" s="140" t="s">
+        <v>469</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A41" s="136">
+      <c r="A41" s="138">
         <v>46143</v>
       </c>
-      <c r="B41" s="138" t="s">
-        <v>369</v>
+      <c r="B41" s="140" t="s">
+        <v>470</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A42" s="136">
+      <c r="A42" s="138">
         <v>46160</v>
       </c>
-      <c r="B42" s="138" t="s">
-        <v>370</v>
+      <c r="B42" s="140" t="s">
+        <v>471</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A43" s="136">
+      <c r="A43" s="138">
         <v>46181</v>
       </c>
-      <c r="B43" s="138" t="s">
-        <v>371</v>
+      <c r="B43" s="140" t="s">
+        <v>472</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A44" s="136">
+      <c r="A44" s="138">
         <v>46188</v>
       </c>
-      <c r="B44" s="138" t="s">
-        <v>381</v>
+      <c r="B44" s="140" t="s">
+        <v>482</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A45" s="136">
+      <c r="A45" s="138">
         <v>46202</v>
       </c>
-      <c r="B45" s="138" t="s">
-        <v>382</v>
+      <c r="B45" s="140" t="s">
+        <v>483</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A46" s="136">
+      <c r="A46" s="138">
         <v>46223</v>
       </c>
-      <c r="B46" s="138" t="s">
-        <v>373</v>
+      <c r="B46" s="140" t="s">
+        <v>474</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A47" s="136">
+      <c r="A47" s="138">
         <v>46241</v>
       </c>
-      <c r="B47" s="138" t="s">
-        <v>374</v>
+      <c r="B47" s="140" t="s">
+        <v>475</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A48" s="136">
+      <c r="A48" s="138">
         <v>46251</v>
       </c>
-      <c r="B48" s="138" t="s">
-        <v>375</v>
+      <c r="B48" s="140" t="s">
+        <v>476</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A49" s="136">
+      <c r="A49" s="138">
         <v>46307</v>
       </c>
-      <c r="B49" s="138" t="s">
-        <v>376</v>
+      <c r="B49" s="140" t="s">
+        <v>477</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A50" s="136">
+      <c r="A50" s="138">
         <v>46328</v>
       </c>
-      <c r="B50" s="138" t="s">
-        <v>377</v>
+      <c r="B50" s="140" t="s">
+        <v>478</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A51" s="136">
+      <c r="A51" s="138">
         <v>46342</v>
       </c>
-      <c r="B51" s="138" t="s">
-        <v>378</v>
+      <c r="B51" s="140" t="s">
+        <v>479</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A52" s="136">
+      <c r="A52" s="138">
         <v>46364</v>
       </c>
-      <c r="B52" s="138" t="s">
-        <v>379</v>
+      <c r="B52" s="140" t="s">
+        <v>480</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A53" s="136">
+      <c r="A53" s="138">
         <v>46381</v>
       </c>
-      <c r="B53" s="138" t="s">
-        <v>380</v>
+      <c r="B53" s="140" t="s">
+        <v>481</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="17.25" customHeight="1"/>

</xml_diff>

<commit_message>
Actualización de archivos JSON y scripts 17 de junio 2026
</commit_message>
<xml_diff>
--- a/Tuya.xlsx
+++ b/Tuya.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12135"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7455"/>
   </bookViews>
   <sheets>
     <sheet name="EN PROCESO (Tuya)" sheetId="1" r:id="rId1"/>
@@ -1537,7 +1537,7 @@
     <t>Desde seguridad solicitan entregar un informe de uso de pemrisos en el aplicativo de Imagine sobre varios usuarios</t>
   </si>
   <si>
-    <t>04/06/2026: Se realiza reunion con los usuarios para aclarar el alcance de la solicitud</t>
+    <t>04/06/2026: Se realiza reunión con los usuarios para aclarar el alcance de la solicitud.</t>
   </si>
   <si>
     <t xml:space="preserve"> Año Nuevo</t>
@@ -2091,7 +2091,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="141">
+  <cellXfs count="142">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2488,6 +2488,9 @@
     <xf numFmtId="14" fontId="12" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="12" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="14" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -2859,7 +2862,7 @@
       NETWORKDAYS(J2,L2,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="N2" s="21"/>
       <c r="O2" s="21"/>
@@ -2928,7 +2931,7 @@
       NETWORKDAYS(J3,L3,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="N3" s="34"/>
       <c r="O3" s="34"/>
@@ -2999,7 +3002,7 @@
       NETWORKDAYS(J4,L4,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="N4" s="22"/>
       <c r="O4" s="22"/>
@@ -3070,7 +3073,7 @@
       NETWORKDAYS(J5,L5,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="N5" s="34"/>
       <c r="O5" s="34"/>
@@ -3141,7 +3144,7 @@
       NETWORKDAYS(J6,L6,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="N6" s="21"/>
       <c r="O6" s="21"/>
@@ -3212,7 +3215,7 @@
       NETWORKDAYS(J7,L7,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="N7" s="41"/>
       <c r="O7" s="41"/>
@@ -3283,7 +3286,7 @@
       NETWORKDAYS(J8,L8,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="N8" s="22"/>
       <c r="O8" s="22"/>
@@ -3944,7 +3947,7 @@
       NETWORKDAYS(J17,L17,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="N17" s="35"/>
       <c r="O17" s="35"/>
@@ -5256,7 +5259,7 @@
       NETWORKDAYS(J35,L35,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="N35" s="76"/>
       <c r="O35" s="76">
@@ -5842,7 +5845,7 @@
       NETWORKDAYS(J43,L43,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="N43" s="41"/>
       <c r="O43" s="41"/>
@@ -10596,7 +10599,7 @@
       NETWORKDAYS(J107,L107,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="N107" s="41"/>
       <c r="O107" s="41"/>
@@ -12791,8 +12794,8 @@
       <c r="Q136" s="55" t="s">
         <v>446</v>
       </c>
-      <c r="R136" s="133" t="s">
-        <v>39</v>
+      <c r="R136" s="138" t="s">
+        <v>381</v>
       </c>
       <c r="S136" s="109"/>
       <c r="T136" s="110"/>
@@ -12846,426 +12849,426 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A1" s="138">
+      <c r="A1" s="139">
         <v>45292</v>
       </c>
-      <c r="B1" s="139" t="s">
+      <c r="B1" s="140" t="s">
         <v>447</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A2" s="138">
+      <c r="A2" s="139">
         <v>45299</v>
       </c>
-      <c r="B2" s="139" t="s">
+      <c r="B2" s="140" t="s">
         <v>448</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A3" s="138">
+      <c r="A3" s="139">
         <v>45376</v>
       </c>
-      <c r="B3" s="139" t="s">
+      <c r="B3" s="140" t="s">
         <v>449</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A4" s="138">
+      <c r="A4" s="139">
         <v>45379</v>
       </c>
-      <c r="B4" s="139" t="s">
+      <c r="B4" s="140" t="s">
         <v>450</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A5" s="138">
+      <c r="A5" s="139">
         <v>45380</v>
       </c>
-      <c r="B5" s="139" t="s">
+      <c r="B5" s="140" t="s">
         <v>451</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A6" s="138">
+      <c r="A6" s="139">
         <v>45413</v>
       </c>
-      <c r="B6" s="139" t="s">
+      <c r="B6" s="140" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A7" s="138">
+      <c r="A7" s="139">
         <v>45425</v>
       </c>
-      <c r="B7" s="139" t="s">
+      <c r="B7" s="140" t="s">
         <v>453</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A8" s="138">
+      <c r="A8" s="139">
         <v>45446</v>
       </c>
-      <c r="B8" s="139" t="s">
+      <c r="B8" s="140" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A9" s="138">
+      <c r="A9" s="139">
         <v>45453</v>
       </c>
-      <c r="B9" s="139" t="s">
+      <c r="B9" s="140" t="s">
         <v>455</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A10" s="138">
+      <c r="A10" s="139">
         <v>45474</v>
       </c>
-      <c r="B10" s="139" t="s">
+      <c r="B10" s="140" t="s">
         <v>456</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A11" s="138">
+      <c r="A11" s="139">
         <v>45493</v>
       </c>
-      <c r="B11" s="139" t="s">
+      <c r="B11" s="140" t="s">
         <v>457</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A12" s="138">
+      <c r="A12" s="139">
         <v>45511</v>
       </c>
-      <c r="B12" s="139" t="s">
+      <c r="B12" s="140" t="s">
         <v>458</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A13" s="138">
+      <c r="A13" s="139">
         <v>45523</v>
       </c>
-      <c r="B13" s="139" t="s">
+      <c r="B13" s="140" t="s">
         <v>459</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A14" s="138">
+      <c r="A14" s="139">
         <v>45579</v>
       </c>
-      <c r="B14" s="139" t="s">
+      <c r="B14" s="140" t="s">
         <v>460</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A15" s="138">
+      <c r="A15" s="139">
         <v>45600</v>
       </c>
-      <c r="B15" s="139" t="s">
+      <c r="B15" s="140" t="s">
         <v>461</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A16" s="138">
+      <c r="A16" s="139">
         <v>45607</v>
       </c>
-      <c r="B16" s="139" t="s">
+      <c r="B16" s="140" t="s">
         <v>462</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A17" s="138">
+      <c r="A17" s="139">
         <v>45634</v>
       </c>
-      <c r="B17" s="139" t="s">
+      <c r="B17" s="140" t="s">
         <v>463</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A18" s="138">
+      <c r="A18" s="139">
         <v>45651</v>
       </c>
-      <c r="B18" s="139" t="s">
+      <c r="B18" s="140" t="s">
         <v>464</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A19" s="138">
+      <c r="A19" s="139">
         <v>45658</v>
       </c>
-      <c r="B19" s="140" t="s">
+      <c r="B19" s="141" t="s">
         <v>465</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A20" s="138">
+      <c r="A20" s="139">
         <v>45663</v>
       </c>
-      <c r="B20" s="140" t="s">
+      <c r="B20" s="141" t="s">
         <v>466</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A21" s="138">
+      <c r="A21" s="139">
         <v>45740</v>
       </c>
-      <c r="B21" s="140" t="s">
+      <c r="B21" s="141" t="s">
         <v>467</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A22" s="138">
+      <c r="A22" s="139">
         <v>45764</v>
       </c>
-      <c r="B22" s="140" t="s">
+      <c r="B22" s="141" t="s">
         <v>468</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A23" s="138">
+      <c r="A23" s="139">
         <v>45765</v>
       </c>
-      <c r="B23" s="140" t="s">
+      <c r="B23" s="141" t="s">
         <v>469</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A24" s="138">
+      <c r="A24" s="139">
         <v>45778</v>
       </c>
-      <c r="B24" s="140" t="s">
+      <c r="B24" s="141" t="s">
         <v>470</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A25" s="138">
+      <c r="A25" s="139">
         <v>45810</v>
       </c>
-      <c r="B25" s="140" t="s">
+      <c r="B25" s="141" t="s">
         <v>471</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A26" s="138">
+      <c r="A26" s="139">
         <v>45831</v>
       </c>
-      <c r="B26" s="140" t="s">
+      <c r="B26" s="141" t="s">
         <v>472</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A27" s="138">
+      <c r="A27" s="139">
         <v>45838</v>
       </c>
-      <c r="B27" s="140" t="s">
+      <c r="B27" s="141" t="s">
         <v>473</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A28" s="138">
+      <c r="A28" s="139">
         <v>45858</v>
       </c>
-      <c r="B28" s="140" t="s">
+      <c r="B28" s="141" t="s">
         <v>474</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A29" s="138">
+      <c r="A29" s="139">
         <v>45876</v>
       </c>
-      <c r="B29" s="140" t="s">
+      <c r="B29" s="141" t="s">
         <v>475</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A30" s="138">
+      <c r="A30" s="139">
         <v>45887</v>
       </c>
-      <c r="B30" s="140" t="s">
+      <c r="B30" s="141" t="s">
         <v>476</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A31" s="138">
+      <c r="A31" s="139">
         <v>45943</v>
       </c>
-      <c r="B31" s="140" t="s">
+      <c r="B31" s="141" t="s">
         <v>477</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A32" s="138">
+      <c r="A32" s="139">
         <v>45964</v>
       </c>
-      <c r="B32" s="140" t="s">
+      <c r="B32" s="141" t="s">
         <v>478</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A33" s="138">
+      <c r="A33" s="139">
         <v>45978</v>
       </c>
-      <c r="B33" s="140" t="s">
+      <c r="B33" s="141" t="s">
         <v>479</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A34" s="138">
+      <c r="A34" s="139">
         <v>45999</v>
       </c>
-      <c r="B34" s="140" t="s">
+      <c r="B34" s="141" t="s">
         <v>480</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A35" s="138">
+      <c r="A35" s="139">
         <v>46016</v>
       </c>
-      <c r="B35" s="140" t="s">
+      <c r="B35" s="141" t="s">
         <v>481</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A36" s="138">
+      <c r="A36" s="139">
         <v>46023</v>
       </c>
-      <c r="B36" s="140" t="s">
+      <c r="B36" s="141" t="s">
         <v>465</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A37" s="138">
+      <c r="A37" s="139">
         <v>46034</v>
       </c>
-      <c r="B37" s="140" t="s">
+      <c r="B37" s="141" t="s">
         <v>466</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A38" s="138">
+      <c r="A38" s="139">
         <v>46104</v>
       </c>
-      <c r="B38" s="140" t="s">
+      <c r="B38" s="141" t="s">
         <v>467</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A39" s="138">
+      <c r="A39" s="139">
         <v>46114</v>
       </c>
-      <c r="B39" s="140" t="s">
+      <c r="B39" s="141" t="s">
         <v>468</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A40" s="138">
+      <c r="A40" s="139">
         <v>46115</v>
       </c>
-      <c r="B40" s="140" t="s">
+      <c r="B40" s="141" t="s">
         <v>469</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A41" s="138">
+      <c r="A41" s="139">
         <v>46143</v>
       </c>
-      <c r="B41" s="140" t="s">
+      <c r="B41" s="141" t="s">
         <v>470</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A42" s="138">
+      <c r="A42" s="139">
         <v>46160</v>
       </c>
-      <c r="B42" s="140" t="s">
+      <c r="B42" s="141" t="s">
         <v>471</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A43" s="138">
+      <c r="A43" s="139">
         <v>46181</v>
       </c>
-      <c r="B43" s="140" t="s">
+      <c r="B43" s="141" t="s">
         <v>472</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A44" s="138">
+      <c r="A44" s="139">
         <v>46188</v>
       </c>
-      <c r="B44" s="140" t="s">
+      <c r="B44" s="141" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A45" s="138">
+      <c r="A45" s="139">
         <v>46202</v>
       </c>
-      <c r="B45" s="140" t="s">
+      <c r="B45" s="141" t="s">
         <v>483</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A46" s="138">
+      <c r="A46" s="139">
         <v>46223</v>
       </c>
-      <c r="B46" s="140" t="s">
+      <c r="B46" s="141" t="s">
         <v>474</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A47" s="138">
+      <c r="A47" s="139">
         <v>46241</v>
       </c>
-      <c r="B47" s="140" t="s">
+      <c r="B47" s="141" t="s">
         <v>475</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A48" s="138">
+      <c r="A48" s="139">
         <v>46251</v>
       </c>
-      <c r="B48" s="140" t="s">
+      <c r="B48" s="141" t="s">
         <v>476</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A49" s="138">
+      <c r="A49" s="139">
         <v>46307</v>
       </c>
-      <c r="B49" s="140" t="s">
+      <c r="B49" s="141" t="s">
         <v>477</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A50" s="138">
+      <c r="A50" s="139">
         <v>46328</v>
       </c>
-      <c r="B50" s="140" t="s">
+      <c r="B50" s="141" t="s">
         <v>478</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A51" s="138">
+      <c r="A51" s="139">
         <v>46342</v>
       </c>
-      <c r="B51" s="140" t="s">
+      <c r="B51" s="141" t="s">
         <v>479</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A52" s="138">
+      <c r="A52" s="139">
         <v>46364</v>
       </c>
-      <c r="B52" s="140" t="s">
+      <c r="B52" s="141" t="s">
         <v>480</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A53" s="138">
+      <c r="A53" s="139">
         <v>46381</v>
       </c>
-      <c r="B53" s="140" t="s">
+      <c r="B53" s="141" t="s">
         <v>481</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización de archivos JSON y scripts 22 de junio 2026
</commit_message>
<xml_diff>
--- a/Tuya.xlsx
+++ b/Tuya.xlsx
@@ -9,26 +9,26 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7455"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12135"/>
   </bookViews>
   <sheets>
     <sheet name="EN PROCESO (Tuya)" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja2" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'EN PROCESO (Tuya)'!$A$1:$AN$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'EN PROCESO (Tuya)'!$A$1:$AN$138</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="zaziqgNpoVISsllI4B+nz/7Oc9tHu2W8ZCHJjQ2RP7c="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="lvSOJAmnbJl513UOCE1rD7zdD+BjojPjmdJyAbwqJUg="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1002" uniqueCount="484">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1016" uniqueCount="489">
   <si>
     <t>Asignado a</t>
   </si>
@@ -1538,6 +1538,21 @@
   </si>
   <si>
     <t>04/06/2026: Se realiza reunión con los usuarios para aclarar el alcance de la solicitud.</t>
+  </si>
+  <si>
+    <t>396</t>
+  </si>
+  <si>
+    <t>Agendamiento reunión con cliente de seguiimiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19/06/2026: Se asiste a reunión de seguimiento con el cliente </t>
+  </si>
+  <si>
+    <t>395</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19/06/2026: Se realiza validación de caso radicado por el usuario, se da solución </t>
   </si>
   <si>
     <t xml:space="preserve"> Año Nuevo</t>
@@ -2723,7 +2738,7 @@
   <sheetPr>
     <tabColor rgb="FF93C47D"/>
   </sheetPr>
-  <dimension ref="A1:AN136"/>
+  <dimension ref="A1:AN138"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.21875" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -2862,7 +2877,7 @@
       NETWORKDAYS(J2,L2,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="N2" s="21"/>
       <c r="O2" s="21"/>
@@ -2931,7 +2946,7 @@
       NETWORKDAYS(J3,L3,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="N3" s="34"/>
       <c r="O3" s="34"/>
@@ -3002,7 +3017,7 @@
       NETWORKDAYS(J4,L4,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="N4" s="22"/>
       <c r="O4" s="22"/>
@@ -3073,7 +3088,7 @@
       NETWORKDAYS(J5,L5,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="N5" s="34"/>
       <c r="O5" s="34"/>
@@ -3144,7 +3159,7 @@
       NETWORKDAYS(J6,L6,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="N6" s="21"/>
       <c r="O6" s="21"/>
@@ -3215,7 +3230,7 @@
       NETWORKDAYS(J7,L7,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="N7" s="41"/>
       <c r="O7" s="41"/>
@@ -3286,7 +3301,7 @@
       NETWORKDAYS(J8,L8,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="N8" s="22"/>
       <c r="O8" s="22"/>
@@ -3947,7 +3962,7 @@
       NETWORKDAYS(J17,L17,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="N17" s="35"/>
       <c r="O17" s="35"/>
@@ -5259,7 +5274,7 @@
       NETWORKDAYS(J35,L35,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="N35" s="76"/>
       <c r="O35" s="76">
@@ -5845,7 +5860,7 @@
       NETWORKDAYS(J43,L43,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="N43" s="41"/>
       <c r="O43" s="41"/>
@@ -10599,7 +10614,7 @@
       NETWORKDAYS(J107,L107,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="N107" s="41"/>
       <c r="O107" s="41"/>
@@ -12795,7 +12810,7 @@
         <v>446</v>
       </c>
       <c r="R136" s="138" t="s">
-        <v>381</v>
+        <v>39</v>
       </c>
       <c r="S136" s="109"/>
       <c r="T136" s="110"/>
@@ -12820,18 +12835,168 @@
       <c r="AM136" s="110"/>
       <c r="AN136" s="111"/>
     </row>
+    <row r="137" spans="1:40">
+      <c r="A137" s="112" t="s">
+        <v>25</v>
+      </c>
+      <c r="B137" s="130" t="s">
+        <v>447</v>
+      </c>
+      <c r="C137" s="84" t="s">
+        <v>282</v>
+      </c>
+      <c r="D137" s="90" t="s">
+        <v>448</v>
+      </c>
+      <c r="E137" s="95"/>
+      <c r="F137" s="101" t="s">
+        <v>46</v>
+      </c>
+      <c r="G137" s="102">
+        <v>100</v>
+      </c>
+      <c r="H137" s="33">
+        <f>IF(OR(J137="",K137="",K137&lt;J137),0,NETWORKDAYS(J137,K137,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I137" s="76">
+        <v>46191</v>
+      </c>
+      <c r="J137" s="76">
+        <v>46191</v>
+      </c>
+      <c r="K137" s="41"/>
+      <c r="L137" s="76">
+        <v>46191</v>
+      </c>
+      <c r="M137" s="36">
+        <f ca="1">IF(OR(J137="",AND(L137="",TODAY()&lt;J137),AND(L137&lt;&gt;"",L137&lt;J137)),0,
+   IF(L137="",
+      NETWORKDAYS(J137,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J137,L137,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N137" s="41"/>
+      <c r="O137" s="41"/>
+      <c r="P137" s="41"/>
+      <c r="Q137" s="92" t="s">
+        <v>449</v>
+      </c>
+      <c r="R137" s="133" t="s">
+        <v>39</v>
+      </c>
+      <c r="S137" s="106"/>
+      <c r="T137" s="107"/>
+      <c r="U137" s="107"/>
+      <c r="V137" s="107"/>
+      <c r="W137" s="107"/>
+      <c r="X137" s="107"/>
+      <c r="Y137" s="107"/>
+      <c r="Z137" s="107"/>
+      <c r="AA137" s="107"/>
+      <c r="AB137" s="107"/>
+      <c r="AC137" s="107"/>
+      <c r="AD137" s="107"/>
+      <c r="AE137" s="107"/>
+      <c r="AF137" s="107"/>
+      <c r="AG137" s="107"/>
+      <c r="AH137" s="107"/>
+      <c r="AI137" s="107"/>
+      <c r="AJ137" s="107"/>
+      <c r="AK137" s="107"/>
+      <c r="AL137" s="107"/>
+      <c r="AM137" s="107"/>
+      <c r="AN137" s="108"/>
+    </row>
+    <row r="138" spans="1:40">
+      <c r="A138" s="116" t="s">
+        <v>25</v>
+      </c>
+      <c r="B138" s="134" t="s">
+        <v>450</v>
+      </c>
+      <c r="C138" s="87" t="s">
+        <v>204</v>
+      </c>
+      <c r="D138" s="91" t="s">
+        <v>390</v>
+      </c>
+      <c r="E138" s="93"/>
+      <c r="F138" s="103" t="s">
+        <v>46</v>
+      </c>
+      <c r="G138" s="104">
+        <v>100</v>
+      </c>
+      <c r="H138" s="20">
+        <f>IF(OR(J138="",K138="",K138&lt;J138),0,NETWORKDAYS(J138,K138,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I138" s="68">
+        <v>46192</v>
+      </c>
+      <c r="J138" s="68">
+        <v>46192</v>
+      </c>
+      <c r="K138" s="44"/>
+      <c r="L138" s="68">
+        <v>46192</v>
+      </c>
+      <c r="M138" s="23">
+        <f ca="1">IF(OR(J138="",AND(L138="",TODAY()&lt;J138),AND(L138&lt;&gt;"",L138&lt;J138)),0,
+   IF(L138="",
+      NETWORKDAYS(J138,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J138,L138,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N138" s="44"/>
+      <c r="O138" s="44"/>
+      <c r="P138" s="44"/>
+      <c r="Q138" s="55" t="s">
+        <v>451</v>
+      </c>
+      <c r="R138" s="129" t="s">
+        <v>39</v>
+      </c>
+      <c r="S138" s="109"/>
+      <c r="T138" s="110"/>
+      <c r="U138" s="110"/>
+      <c r="V138" s="110"/>
+      <c r="W138" s="110"/>
+      <c r="X138" s="110"/>
+      <c r="Y138" s="110"/>
+      <c r="Z138" s="110"/>
+      <c r="AA138" s="110"/>
+      <c r="AB138" s="110"/>
+      <c r="AC138" s="110"/>
+      <c r="AD138" s="110"/>
+      <c r="AE138" s="110"/>
+      <c r="AF138" s="110"/>
+      <c r="AG138" s="110"/>
+      <c r="AH138" s="110"/>
+      <c r="AI138" s="110"/>
+      <c r="AJ138" s="110"/>
+      <c r="AK138" s="110"/>
+      <c r="AL138" s="110"/>
+      <c r="AM138" s="110"/>
+      <c r="AN138" s="111"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AN136"/>
-  <conditionalFormatting sqref="B2:B136">
+  <autoFilter ref="A1:AN138"/>
+  <conditionalFormatting sqref="B2:B138">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>COUNTIF(B$2:B$16,B2)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="I2:L9 J10:L10 I11:L54 N2:P54 I56:L136 N56:P136">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="I2:L9 J10:L10 I11:L54 N2:P54 I56:L138 N56:P138">
       <formula1>OR(NOT(ISERROR(DATEVALUE(I2))), AND(ISNUMBER(I2), LEFT(CELL("format", I2))="D"))</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F136">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F138">
       <formula1>"FINALIZADO,EN PROCESO,PAUSADO,EN TEST,PENDIENTE,PRUEBAS CLIENTE,PRUEBAS IMAGINE,PASO A PRODUCCION"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12853,7 +13018,7 @@
         <v>45292</v>
       </c>
       <c r="B1" s="140" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="17.25" customHeight="1">
@@ -12861,7 +13026,7 @@
         <v>45299</v>
       </c>
       <c r="B2" s="140" t="s">
-        <v>448</v>
+        <v>453</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="17.25" customHeight="1">
@@ -12869,7 +13034,7 @@
         <v>45376</v>
       </c>
       <c r="B3" s="140" t="s">
-        <v>449</v>
+        <v>454</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="17.25" customHeight="1">
@@ -12877,7 +13042,7 @@
         <v>45379</v>
       </c>
       <c r="B4" s="140" t="s">
-        <v>450</v>
+        <v>455</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="17.25" customHeight="1">
@@ -12885,7 +13050,7 @@
         <v>45380</v>
       </c>
       <c r="B5" s="140" t="s">
-        <v>451</v>
+        <v>456</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="17.25" customHeight="1">
@@ -12893,7 +13058,7 @@
         <v>45413</v>
       </c>
       <c r="B6" s="140" t="s">
-        <v>452</v>
+        <v>457</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="17.25" customHeight="1">
@@ -12901,7 +13066,7 @@
         <v>45425</v>
       </c>
       <c r="B7" s="140" t="s">
-        <v>453</v>
+        <v>458</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="17.25" customHeight="1">
@@ -12909,7 +13074,7 @@
         <v>45446</v>
       </c>
       <c r="B8" s="140" t="s">
-        <v>454</v>
+        <v>459</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="17.25" customHeight="1">
@@ -12917,7 +13082,7 @@
         <v>45453</v>
       </c>
       <c r="B9" s="140" t="s">
-        <v>455</v>
+        <v>460</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="17.25" customHeight="1">
@@ -12925,7 +13090,7 @@
         <v>45474</v>
       </c>
       <c r="B10" s="140" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="17.25" customHeight="1">
@@ -12933,7 +13098,7 @@
         <v>45493</v>
       </c>
       <c r="B11" s="140" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="17.25" customHeight="1">
@@ -12941,7 +13106,7 @@
         <v>45511</v>
       </c>
       <c r="B12" s="140" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="17.25" customHeight="1">
@@ -12949,7 +13114,7 @@
         <v>45523</v>
       </c>
       <c r="B13" s="140" t="s">
-        <v>459</v>
+        <v>464</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="17.25" customHeight="1">
@@ -12957,7 +13122,7 @@
         <v>45579</v>
       </c>
       <c r="B14" s="140" t="s">
-        <v>460</v>
+        <v>465</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="17.25" customHeight="1">
@@ -12965,7 +13130,7 @@
         <v>45600</v>
       </c>
       <c r="B15" s="140" t="s">
-        <v>461</v>
+        <v>466</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="17.25" customHeight="1">
@@ -12973,7 +13138,7 @@
         <v>45607</v>
       </c>
       <c r="B16" s="140" t="s">
-        <v>462</v>
+        <v>467</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="17.25" customHeight="1">
@@ -12981,7 +13146,7 @@
         <v>45634</v>
       </c>
       <c r="B17" s="140" t="s">
-        <v>463</v>
+        <v>468</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="17.25" customHeight="1">
@@ -12989,7 +13154,7 @@
         <v>45651</v>
       </c>
       <c r="B18" s="140" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="17.25" customHeight="1">
@@ -12997,7 +13162,7 @@
         <v>45658</v>
       </c>
       <c r="B19" s="141" t="s">
-        <v>465</v>
+        <v>470</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="17.25" customHeight="1">
@@ -13005,7 +13170,7 @@
         <v>45663</v>
       </c>
       <c r="B20" s="141" t="s">
-        <v>466</v>
+        <v>471</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="17.25" customHeight="1">
@@ -13013,7 +13178,7 @@
         <v>45740</v>
       </c>
       <c r="B21" s="141" t="s">
-        <v>467</v>
+        <v>472</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="17.25" customHeight="1">
@@ -13021,7 +13186,7 @@
         <v>45764</v>
       </c>
       <c r="B22" s="141" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="17.25" customHeight="1">
@@ -13029,7 +13194,7 @@
         <v>45765</v>
       </c>
       <c r="B23" s="141" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="17.25" customHeight="1">
@@ -13037,7 +13202,7 @@
         <v>45778</v>
       </c>
       <c r="B24" s="141" t="s">
-        <v>470</v>
+        <v>475</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="17.25" customHeight="1">
@@ -13045,7 +13210,7 @@
         <v>45810</v>
       </c>
       <c r="B25" s="141" t="s">
-        <v>471</v>
+        <v>476</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="17.25" customHeight="1">
@@ -13053,7 +13218,7 @@
         <v>45831</v>
       </c>
       <c r="B26" s="141" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="17.25" customHeight="1">
@@ -13061,7 +13226,7 @@
         <v>45838</v>
       </c>
       <c r="B27" s="141" t="s">
-        <v>473</v>
+        <v>478</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="17.25" customHeight="1">
@@ -13069,7 +13234,7 @@
         <v>45858</v>
       </c>
       <c r="B28" s="141" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="17.25" customHeight="1">
@@ -13077,7 +13242,7 @@
         <v>45876</v>
       </c>
       <c r="B29" s="141" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="17.25" customHeight="1">
@@ -13085,7 +13250,7 @@
         <v>45887</v>
       </c>
       <c r="B30" s="141" t="s">
-        <v>476</v>
+        <v>481</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="17.25" customHeight="1">
@@ -13093,7 +13258,7 @@
         <v>45943</v>
       </c>
       <c r="B31" s="141" t="s">
-        <v>477</v>
+        <v>482</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="17.25" customHeight="1">
@@ -13101,7 +13266,7 @@
         <v>45964</v>
       </c>
       <c r="B32" s="141" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="17.25" customHeight="1">
@@ -13109,7 +13274,7 @@
         <v>45978</v>
       </c>
       <c r="B33" s="141" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="17.25" customHeight="1">
@@ -13117,7 +13282,7 @@
         <v>45999</v>
       </c>
       <c r="B34" s="141" t="s">
-        <v>480</v>
+        <v>485</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="17.25" customHeight="1">
@@ -13125,7 +13290,7 @@
         <v>46016</v>
       </c>
       <c r="B35" s="141" t="s">
-        <v>481</v>
+        <v>486</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="17.25" customHeight="1">
@@ -13133,7 +13298,7 @@
         <v>46023</v>
       </c>
       <c r="B36" s="141" t="s">
-        <v>465</v>
+        <v>470</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="17.25" customHeight="1">
@@ -13141,7 +13306,7 @@
         <v>46034</v>
       </c>
       <c r="B37" s="141" t="s">
-        <v>466</v>
+        <v>471</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="17.25" customHeight="1">
@@ -13149,7 +13314,7 @@
         <v>46104</v>
       </c>
       <c r="B38" s="141" t="s">
-        <v>467</v>
+        <v>472</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="17.25" customHeight="1">
@@ -13157,7 +13322,7 @@
         <v>46114</v>
       </c>
       <c r="B39" s="141" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="17.25" customHeight="1">
@@ -13165,7 +13330,7 @@
         <v>46115</v>
       </c>
       <c r="B40" s="141" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="17.25" customHeight="1">
@@ -13173,7 +13338,7 @@
         <v>46143</v>
       </c>
       <c r="B41" s="141" t="s">
-        <v>470</v>
+        <v>475</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="17.25" customHeight="1">
@@ -13181,7 +13346,7 @@
         <v>46160</v>
       </c>
       <c r="B42" s="141" t="s">
-        <v>471</v>
+        <v>476</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="17.25" customHeight="1">
@@ -13189,7 +13354,7 @@
         <v>46181</v>
       </c>
       <c r="B43" s="141" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="17.25" customHeight="1">
@@ -13197,7 +13362,7 @@
         <v>46188</v>
       </c>
       <c r="B44" s="141" t="s">
-        <v>482</v>
+        <v>487</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="17.25" customHeight="1">
@@ -13205,7 +13370,7 @@
         <v>46202</v>
       </c>
       <c r="B45" s="141" t="s">
-        <v>483</v>
+        <v>488</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="17.25" customHeight="1">
@@ -13213,7 +13378,7 @@
         <v>46223</v>
       </c>
       <c r="B46" s="141" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="17.25" customHeight="1">
@@ -13221,7 +13386,7 @@
         <v>46241</v>
       </c>
       <c r="B47" s="141" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="17.25" customHeight="1">
@@ -13229,7 +13394,7 @@
         <v>46251</v>
       </c>
       <c r="B48" s="141" t="s">
-        <v>476</v>
+        <v>481</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="17.25" customHeight="1">
@@ -13237,7 +13402,7 @@
         <v>46307</v>
       </c>
       <c r="B49" s="141" t="s">
-        <v>477</v>
+        <v>482</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="17.25" customHeight="1">
@@ -13245,7 +13410,7 @@
         <v>46328</v>
       </c>
       <c r="B50" s="141" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="17.25" customHeight="1">
@@ -13253,7 +13418,7 @@
         <v>46342</v>
       </c>
       <c r="B51" s="141" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="17.25" customHeight="1">
@@ -13261,7 +13426,7 @@
         <v>46364</v>
       </c>
       <c r="B52" s="141" t="s">
-        <v>480</v>
+        <v>485</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="17.25" customHeight="1">
@@ -13269,7 +13434,7 @@
         <v>46381</v>
       </c>
       <c r="B53" s="141" t="s">
-        <v>481</v>
+        <v>486</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="17.25" customHeight="1"/>

</xml_diff>